<commit_message>
APS correção na planilha PV.xlsx
</commit_message>
<xml_diff>
--- a/PV.xlsx
+++ b/PV.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D9F1958-EB96-415B-AF4D-A71F8C14AF78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F4318F-A544-4813-AFB3-5387EDBD918E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,9 +32,6 @@
   </si>
   <si>
     <t>DATA DE ENTREGA</t>
-  </si>
-  <si>
-    <t>QUANTIDADE</t>
   </si>
   <si>
     <t>CORTE - SERRA</t>
@@ -362,6 +359,9 @@
   </si>
   <si>
     <t>25/07/2026</t>
+  </si>
+  <si>
+    <t>QTD</t>
   </si>
 </sst>
 </file>
@@ -767,70 +767,70 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="L1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.3">
@@ -838,13 +838,13 @@
         <v>6549</v>
       </c>
       <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
         <v>26</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>27</v>
-      </c>
-      <c r="D2" t="s">
-        <v>28</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -918,13 +918,13 @@
         <v>6552</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
         <v>27</v>
-      </c>
-      <c r="D3" t="s">
-        <v>28</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -998,13 +998,13 @@
         <v>6764</v>
       </c>
       <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
         <v>30</v>
       </c>
-      <c r="C4" t="s">
-        <v>31</v>
-      </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E4">
         <v>4</v>
@@ -1078,13 +1078,13 @@
         <v>6780</v>
       </c>
       <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
         <v>32</v>
       </c>
-      <c r="C5" t="s">
-        <v>33</v>
-      </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E5">
         <v>14</v>
@@ -1158,13 +1158,13 @@
         <v>6873</v>
       </c>
       <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
         <v>34</v>
       </c>
-      <c r="C6" t="s">
-        <v>35</v>
-      </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E6">
         <v>3</v>
@@ -1238,13 +1238,13 @@
         <v>6550</v>
       </c>
       <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -1318,13 +1318,13 @@
         <v>6553</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -1401,10 +1401,10 @@
         <v>15967961</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E9">
         <v>102</v>
@@ -1478,13 +1478,13 @@
         <v>6710</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E10">
         <v>146</v>
@@ -1561,10 +1561,10 @@
         <v>14558705</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E11">
         <v>3</v>
@@ -1641,10 +1641,10 @@
         <v>13991667</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E12">
         <v>27</v>
@@ -1721,10 +1721,10 @@
         <v>13991819</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E13">
         <v>30</v>
@@ -1801,10 +1801,10 @@
         <v>13991818</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E14">
         <v>9</v>
@@ -1881,10 +1881,10 @@
         <v>11469602</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E15">
         <v>48</v>
@@ -1961,10 +1961,10 @@
         <v>13319685</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E16">
         <v>12</v>
@@ -2041,10 +2041,10 @@
         <v>12421834</v>
       </c>
       <c r="C17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E17">
         <v>18</v>
@@ -2121,10 +2121,10 @@
         <v>15976733</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E18">
         <v>87</v>
@@ -2201,10 +2201,10 @@
         <v>15976244</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E19">
         <v>87</v>
@@ -2281,10 +2281,10 @@
         <v>14140591</v>
       </c>
       <c r="C20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E20">
         <v>30</v>
@@ -2361,10 +2361,10 @@
         <v>13991909</v>
       </c>
       <c r="C21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E21">
         <v>9</v>
@@ -2441,10 +2441,10 @@
         <v>13991663</v>
       </c>
       <c r="C22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E22">
         <v>9</v>
@@ -2521,10 +2521,10 @@
         <v>13588930</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E23">
         <v>18</v>
@@ -2601,10 +2601,10 @@
         <v>14577954</v>
       </c>
       <c r="C24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D24" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E24">
         <v>3</v>
@@ -2681,10 +2681,10 @@
         <v>14577949</v>
       </c>
       <c r="C25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E25">
         <v>3</v>
@@ -2761,10 +2761,10 @@
         <v>11468826</v>
       </c>
       <c r="C26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D26" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E26">
         <v>24</v>
@@ -2841,10 +2841,10 @@
         <v>11468775</v>
       </c>
       <c r="C27" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E27">
         <v>24</v>
@@ -2921,10 +2921,10 @@
         <v>11468114</v>
       </c>
       <c r="C28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D28" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E28">
         <v>24</v>
@@ -3001,10 +3001,10 @@
         <v>11467111</v>
       </c>
       <c r="C29" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D29" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E29">
         <v>24</v>
@@ -3078,13 +3078,13 @@
         <v>6842</v>
       </c>
       <c r="B30" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" t="s">
+        <v>30</v>
+      </c>
+      <c r="D30" t="s">
         <v>39</v>
-      </c>
-      <c r="C30" t="s">
-        <v>31</v>
-      </c>
-      <c r="D30" t="s">
-        <v>40</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -3158,13 +3158,13 @@
         <v>6859</v>
       </c>
       <c r="B31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" t="s">
+        <v>32</v>
+      </c>
+      <c r="D31" t="s">
         <v>41</v>
-      </c>
-      <c r="C31" t="s">
-        <v>33</v>
-      </c>
-      <c r="D31" t="s">
-        <v>42</v>
       </c>
       <c r="E31">
         <v>6</v>
@@ -3238,13 +3238,13 @@
         <v>6519</v>
       </c>
       <c r="B32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" t="s">
+        <v>30</v>
+      </c>
+      <c r="D32" t="s">
         <v>43</v>
-      </c>
-      <c r="C32" t="s">
-        <v>31</v>
-      </c>
-      <c r="D32" t="s">
-        <v>44</v>
       </c>
       <c r="E32">
         <v>28</v>
@@ -3318,13 +3318,13 @@
         <v>6870</v>
       </c>
       <c r="B33" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D33" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E33">
         <v>2</v>
@@ -3398,13 +3398,13 @@
         <v>6875</v>
       </c>
       <c r="B34" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D34" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E34">
         <v>15</v>
@@ -3478,13 +3478,13 @@
         <v>6953</v>
       </c>
       <c r="B35" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C35" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D35" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E35">
         <v>4</v>
@@ -3495,13 +3495,13 @@
         <v>6013</v>
       </c>
       <c r="B36" t="s">
+        <v>47</v>
+      </c>
+      <c r="C36" t="s">
         <v>48</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>49</v>
-      </c>
-      <c r="D36" t="s">
-        <v>50</v>
       </c>
       <c r="E36">
         <v>500</v>
@@ -3575,13 +3575,13 @@
         <v>6522</v>
       </c>
       <c r="B37" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D37" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E37">
         <v>16</v>
@@ -3655,13 +3655,13 @@
         <v>6797</v>
       </c>
       <c r="B38" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C38" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D38" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E38">
         <v>4</v>
@@ -3735,13 +3735,13 @@
         <v>6798</v>
       </c>
       <c r="B39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C39" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E39">
         <v>7</v>
@@ -3815,13 +3815,13 @@
         <v>6827</v>
       </c>
       <c r="B40" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C40" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -3895,13 +3895,13 @@
         <v>6830</v>
       </c>
       <c r="B41" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D41" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E41">
         <v>10</v>
@@ -3975,13 +3975,13 @@
         <v>6754</v>
       </c>
       <c r="B42" t="s">
+        <v>54</v>
+      </c>
+      <c r="C42" t="s">
+        <v>30</v>
+      </c>
+      <c r="D42" t="s">
         <v>55</v>
-      </c>
-      <c r="C42" t="s">
-        <v>31</v>
-      </c>
-      <c r="D42" t="s">
-        <v>56</v>
       </c>
       <c r="E42">
         <v>7</v>
@@ -4055,13 +4055,13 @@
         <v>6942</v>
       </c>
       <c r="B43" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C43" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D43" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -4138,10 +4138,10 @@
         <v>15970137</v>
       </c>
       <c r="C44" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D44" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E44">
         <v>21</v>
@@ -4218,10 +4218,10 @@
         <v>14153893</v>
       </c>
       <c r="C45" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D45" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E45">
         <v>24</v>
@@ -4298,10 +4298,10 @@
         <v>14085079</v>
       </c>
       <c r="C46" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D46" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E46">
         <v>12</v>
@@ -4378,10 +4378,10 @@
         <v>14627922</v>
       </c>
       <c r="C47" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D47" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E47">
         <v>12</v>
@@ -4458,10 +4458,10 @@
         <v>14035990</v>
       </c>
       <c r="C48" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D48" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E48">
         <v>3</v>
@@ -4538,10 +4538,10 @@
         <v>14624464</v>
       </c>
       <c r="C49" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D49" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E49">
         <v>24</v>
@@ -4618,10 +4618,10 @@
         <v>14613011</v>
       </c>
       <c r="C50" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D50" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E50">
         <v>48</v>
@@ -4698,10 +4698,10 @@
         <v>11510278</v>
       </c>
       <c r="C51" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D51" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E51">
         <v>100</v>
@@ -4778,10 +4778,10 @@
         <v>15975246</v>
       </c>
       <c r="C52" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D52" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E52">
         <v>54</v>
@@ -4858,10 +4858,10 @@
         <v>15973874</v>
       </c>
       <c r="C53" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D53" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E53">
         <v>27</v>
@@ -4938,10 +4938,10 @@
         <v>15972626</v>
       </c>
       <c r="C54" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D54" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E54">
         <v>27</v>
@@ -5018,10 +5018,10 @@
         <v>15972619</v>
       </c>
       <c r="C55" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D55" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E55">
         <v>27</v>
@@ -5098,10 +5098,10 @@
         <v>15972293</v>
       </c>
       <c r="C56" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D56" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E56">
         <v>54</v>
@@ -5178,10 +5178,10 @@
         <v>15972104</v>
       </c>
       <c r="C57" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D57" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E57">
         <v>54</v>
@@ -5258,10 +5258,10 @@
         <v>15971930</v>
       </c>
       <c r="C58" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D58" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E58">
         <v>27</v>
@@ -5338,10 +5338,10 @@
         <v>14095131</v>
       </c>
       <c r="C59" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D59" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E59">
         <v>12</v>
@@ -5418,10 +5418,10 @@
         <v>14084370</v>
       </c>
       <c r="C60" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D60" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E60">
         <v>12</v>
@@ -5498,10 +5498,10 @@
         <v>15790045</v>
       </c>
       <c r="C61" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D61" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E61">
         <v>6</v>
@@ -5578,10 +5578,10 @@
         <v>15790121</v>
       </c>
       <c r="C62" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D62" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E62">
         <v>3</v>
@@ -5658,10 +5658,10 @@
         <v>15790046</v>
       </c>
       <c r="C63" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D63" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E63">
         <v>3</v>
@@ -5738,10 +5738,10 @@
         <v>14563966</v>
       </c>
       <c r="C64" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D64" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E64">
         <v>6</v>
@@ -5818,10 +5818,10 @@
         <v>14563925</v>
       </c>
       <c r="C65" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D65" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E65">
         <v>6</v>
@@ -5898,10 +5898,10 @@
         <v>15540457</v>
       </c>
       <c r="C66" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D66" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E66">
         <v>6</v>
@@ -5978,10 +5978,10 @@
         <v>15540450</v>
       </c>
       <c r="C67" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D67" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E67">
         <v>6</v>
@@ -6058,10 +6058,10 @@
         <v>15494648</v>
       </c>
       <c r="C68" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D68" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E68">
         <v>6</v>
@@ -6138,10 +6138,10 @@
         <v>11463275</v>
       </c>
       <c r="C69" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D69" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E69">
         <v>6</v>
@@ -6218,10 +6218,10 @@
         <v>11463274</v>
       </c>
       <c r="C70" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D70" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E70">
         <v>6</v>
@@ -6298,10 +6298,10 @@
         <v>11460670</v>
       </c>
       <c r="C71" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D71" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E71">
         <v>6</v>
@@ -6378,10 +6378,10 @@
         <v>11458375</v>
       </c>
       <c r="C72" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D72" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E72">
         <v>6</v>
@@ -6458,10 +6458,10 @@
         <v>11460314</v>
       </c>
       <c r="C73" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D73" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E73">
         <v>6</v>
@@ -6538,10 +6538,10 @@
         <v>13833429</v>
       </c>
       <c r="C74" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D74" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E74">
         <v>6</v>
@@ -6618,10 +6618,10 @@
         <v>11510278</v>
       </c>
       <c r="C75" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D75" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E75">
         <v>100</v>
@@ -6695,13 +6695,13 @@
         <v>6767</v>
       </c>
       <c r="B76" t="s">
+        <v>58</v>
+      </c>
+      <c r="C76" t="s">
+        <v>30</v>
+      </c>
+      <c r="D76" t="s">
         <v>59</v>
-      </c>
-      <c r="C76" t="s">
-        <v>31</v>
-      </c>
-      <c r="D76" t="s">
-        <v>60</v>
       </c>
       <c r="E76">
         <v>2</v>
@@ -6775,13 +6775,13 @@
         <v>6770</v>
       </c>
       <c r="B77" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C77" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D77" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E77">
         <v>62</v>
@@ -6855,13 +6855,13 @@
         <v>6828</v>
       </c>
       <c r="B78" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C78" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D78" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E78">
         <v>51</v>
@@ -6935,13 +6935,13 @@
         <v>6547</v>
       </c>
       <c r="B79" t="s">
+        <v>25</v>
+      </c>
+      <c r="C79" t="s">
         <v>26</v>
       </c>
-      <c r="C79" t="s">
-        <v>27</v>
-      </c>
       <c r="D79" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -7015,13 +7015,13 @@
         <v>6554</v>
       </c>
       <c r="B80" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C80" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D80" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -7095,13 +7095,13 @@
         <v>6814</v>
       </c>
       <c r="B81" t="s">
+        <v>63</v>
+      </c>
+      <c r="C81" t="s">
+        <v>30</v>
+      </c>
+      <c r="D81" t="s">
         <v>64</v>
-      </c>
-      <c r="C81" t="s">
-        <v>31</v>
-      </c>
-      <c r="D81" t="s">
-        <v>65</v>
       </c>
       <c r="E81">
         <v>3</v>
@@ -7178,10 +7178,10 @@
         <v>15970137</v>
       </c>
       <c r="C82" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D82" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E82">
         <v>24</v>
@@ -7258,10 +7258,10 @@
         <v>15967961</v>
       </c>
       <c r="C83" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D83" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E83">
         <v>123</v>
@@ -7335,13 +7335,13 @@
         <v>6788</v>
       </c>
       <c r="B84" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C84" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D84" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E84">
         <v>8</v>
@@ -7415,13 +7415,13 @@
         <v>6793</v>
       </c>
       <c r="B85" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C85" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D85" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E85">
         <v>4</v>
@@ -7495,13 +7495,13 @@
         <v>6799</v>
       </c>
       <c r="B86" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C86" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D86" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E86">
         <v>3</v>
@@ -7578,10 +7578,10 @@
         <v>11893661</v>
       </c>
       <c r="C87" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D87" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E87">
         <v>36</v>
@@ -7658,10 +7658,10 @@
         <v>14496774</v>
       </c>
       <c r="C88" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D88" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E88">
         <v>9</v>
@@ -7738,10 +7738,10 @@
         <v>17800490</v>
       </c>
       <c r="C89" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D89" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E89">
         <v>9</v>
@@ -7818,10 +7818,10 @@
         <v>14504560</v>
       </c>
       <c r="C90" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D90" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E90">
         <v>9</v>
@@ -7898,10 +7898,10 @@
         <v>17797436</v>
       </c>
       <c r="C91" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D91" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E91">
         <v>6</v>
@@ -7975,13 +7975,13 @@
         <v>6846</v>
       </c>
       <c r="B92" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C92" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D92" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E92">
         <v>9</v>
@@ -8058,10 +8058,10 @@
         <v>13829680</v>
       </c>
       <c r="C93" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D93" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E93">
         <v>6</v>
@@ -8138,10 +8138,10 @@
         <v>13592346</v>
       </c>
       <c r="C94" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D94" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E94">
         <v>6</v>
@@ -8218,10 +8218,10 @@
         <v>15982393</v>
       </c>
       <c r="C95" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D95" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E95">
         <v>3</v>
@@ -8298,10 +8298,10 @@
         <v>13828817</v>
       </c>
       <c r="C96" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D96" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E96">
         <v>6</v>
@@ -8378,10 +8378,10 @@
         <v>16727617</v>
       </c>
       <c r="C97" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D97" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E97">
         <v>20</v>
@@ -8458,10 +8458,10 @@
         <v>11440086</v>
       </c>
       <c r="C98" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D98" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E98">
         <v>10</v>
@@ -8538,10 +8538,10 @@
         <v>13832165</v>
       </c>
       <c r="C99" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D99" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E99">
         <v>6</v>
@@ -8618,10 +8618,10 @@
         <v>12420856</v>
       </c>
       <c r="C100" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D100" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E100">
         <v>6</v>
@@ -8698,10 +8698,10 @@
         <v>12420855</v>
       </c>
       <c r="C101" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D101" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E101">
         <v>6</v>
@@ -8778,10 +8778,10 @@
         <v>12406511</v>
       </c>
       <c r="C102" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D102" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E102">
         <v>12</v>
@@ -8858,10 +8858,10 @@
         <v>12406391</v>
       </c>
       <c r="C103" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D103" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E103">
         <v>6</v>
@@ -8938,10 +8938,10 @@
         <v>16406069</v>
       </c>
       <c r="C104" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D104" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E104">
         <v>3</v>
@@ -9015,13 +9015,13 @@
         <v>6765</v>
       </c>
       <c r="B105" t="s">
+        <v>69</v>
+      </c>
+      <c r="C105" t="s">
+        <v>30</v>
+      </c>
+      <c r="D105" t="s">
         <v>70</v>
-      </c>
-      <c r="C105" t="s">
-        <v>31</v>
-      </c>
-      <c r="D105" t="s">
-        <v>71</v>
       </c>
       <c r="E105">
         <v>2</v>
@@ -9095,13 +9095,13 @@
         <v>6839</v>
       </c>
       <c r="B106" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C106" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D106" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E106">
         <v>3</v>
@@ -9175,13 +9175,13 @@
         <v>6637</v>
       </c>
       <c r="B107" t="s">
+        <v>72</v>
+      </c>
+      <c r="C107" t="s">
+        <v>30</v>
+      </c>
+      <c r="D107" t="s">
         <v>73</v>
-      </c>
-      <c r="C107" t="s">
-        <v>31</v>
-      </c>
-      <c r="D107" t="s">
-        <v>74</v>
       </c>
       <c r="E107">
         <v>10</v>
@@ -9255,13 +9255,13 @@
         <v>6766</v>
       </c>
       <c r="B108" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C108" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D108" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E108">
         <v>7</v>
@@ -9335,13 +9335,13 @@
         <v>6784</v>
       </c>
       <c r="B109" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C109" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D109" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E109">
         <v>200</v>
@@ -9415,13 +9415,13 @@
         <v>6843</v>
       </c>
       <c r="B110" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C110" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D110" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E110">
         <v>4</v>
@@ -9495,13 +9495,13 @@
         <v>6941</v>
       </c>
       <c r="B111" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C111" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D111" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -9575,13 +9575,13 @@
         <v>6786</v>
       </c>
       <c r="B112" t="s">
+        <v>76</v>
+      </c>
+      <c r="C112" t="s">
+        <v>30</v>
+      </c>
+      <c r="D112" t="s">
         <v>77</v>
-      </c>
-      <c r="C112" t="s">
-        <v>31</v>
-      </c>
-      <c r="D112" t="s">
-        <v>78</v>
       </c>
       <c r="E112">
         <v>5</v>
@@ -9658,10 +9658,10 @@
         <v>12864933</v>
       </c>
       <c r="C113" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D113" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E113">
         <v>18</v>
@@ -9738,10 +9738,10 @@
         <v>11510278</v>
       </c>
       <c r="C114" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D114" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E114">
         <v>50</v>
@@ -9818,10 +9818,10 @@
         <v>15494649</v>
       </c>
       <c r="C115" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D115" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E115">
         <v>6</v>
@@ -9898,10 +9898,10 @@
         <v>14494848</v>
       </c>
       <c r="C116" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D116" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E116">
         <v>6</v>
@@ -9978,10 +9978,10 @@
         <v>13279123</v>
       </c>
       <c r="C117" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D117" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E117">
         <v>6</v>
@@ -10058,10 +10058,10 @@
         <v>13202650</v>
       </c>
       <c r="C118" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D118" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E118">
         <v>6</v>
@@ -10138,10 +10138,10 @@
         <v>13993039</v>
       </c>
       <c r="C119" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D119" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E119">
         <v>6</v>
@@ -10218,10 +10218,10 @@
         <v>15481651</v>
       </c>
       <c r="C120" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D120" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E120">
         <v>12</v>
@@ -10298,10 +10298,10 @@
         <v>13319535</v>
       </c>
       <c r="C121" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D121" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E121">
         <v>6</v>
@@ -10375,13 +10375,13 @@
         <v>6640</v>
       </c>
       <c r="B122" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C122" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D122" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E122">
         <v>3</v>
@@ -10455,13 +10455,13 @@
         <v>6641</v>
       </c>
       <c r="B123" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C123" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D123" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E123">
         <v>6</v>
@@ -10535,13 +10535,13 @@
         <v>6885</v>
       </c>
       <c r="B124" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C124" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D124" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E124">
         <v>50</v>
@@ -10615,13 +10615,13 @@
         <v>6831</v>
       </c>
       <c r="B125" t="s">
+        <v>80</v>
+      </c>
+      <c r="C125" t="s">
+        <v>30</v>
+      </c>
+      <c r="D125" t="s">
         <v>81</v>
-      </c>
-      <c r="C125" t="s">
-        <v>31</v>
-      </c>
-      <c r="D125" t="s">
-        <v>82</v>
       </c>
       <c r="E125">
         <v>9</v>
@@ -10698,10 +10698,10 @@
         <v>13828817</v>
       </c>
       <c r="C126" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D126" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E126">
         <v>18</v>
@@ -10778,10 +10778,10 @@
         <v>15967965</v>
       </c>
       <c r="C127" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D127" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E127">
         <v>39</v>
@@ -10858,10 +10858,10 @@
         <v>13832165</v>
       </c>
       <c r="C128" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D128" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E128">
         <v>18</v>
@@ -10938,10 +10938,10 @@
         <v>14085079</v>
       </c>
       <c r="C129" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D129" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E129">
         <v>6</v>
@@ -11018,10 +11018,10 @@
         <v>14153893</v>
       </c>
       <c r="C130" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D130" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E130">
         <v>57</v>
@@ -11098,10 +11098,10 @@
         <v>15970137</v>
       </c>
       <c r="C131" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D131" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E131">
         <v>21</v>
@@ -11178,10 +11178,10 @@
         <v>16110881</v>
       </c>
       <c r="C132" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D132" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E132">
         <v>624</v>
@@ -11258,10 +11258,10 @@
         <v>13991819</v>
       </c>
       <c r="C133" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D133" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E133">
         <v>27</v>
@@ -11338,10 +11338,10 @@
         <v>14060692</v>
       </c>
       <c r="C134" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D134" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E134">
         <v>21</v>
@@ -11418,10 +11418,10 @@
         <v>13588930</v>
       </c>
       <c r="C135" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D135" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E135">
         <v>60</v>
@@ -11498,10 +11498,10 @@
         <v>16727617</v>
       </c>
       <c r="C136" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D136" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E136">
         <v>50</v>
@@ -11578,10 +11578,10 @@
         <v>17800490</v>
       </c>
       <c r="C137" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D137" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E137">
         <v>15</v>
@@ -11658,10 +11658,10 @@
         <v>14504560</v>
       </c>
       <c r="C138" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D138" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E138">
         <v>15</v>
@@ -11738,10 +11738,10 @@
         <v>11893661</v>
       </c>
       <c r="C139" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D139" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E139">
         <v>72</v>
@@ -11818,10 +11818,10 @@
         <v>13833429</v>
       </c>
       <c r="C140" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D140" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E140">
         <v>18</v>
@@ -11898,10 +11898,10 @@
         <v>14494848</v>
       </c>
       <c r="C141" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D141" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E141">
         <v>21</v>
@@ -11978,10 +11978,10 @@
         <v>14354620</v>
       </c>
       <c r="C142" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D142" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E142">
         <v>6</v>
@@ -12058,10 +12058,10 @@
         <v>13991667</v>
       </c>
       <c r="C143" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D143" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E143">
         <v>33</v>
@@ -12138,10 +12138,10 @@
         <v>17797436</v>
       </c>
       <c r="C144" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D144" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E144">
         <v>3</v>
@@ -12218,10 +12218,10 @@
         <v>16110422</v>
       </c>
       <c r="C145" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D145" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E145">
         <v>78</v>
@@ -12298,10 +12298,10 @@
         <v>14496774</v>
       </c>
       <c r="C146" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D146" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E146">
         <v>15</v>
@@ -12375,13 +12375,13 @@
         <v>6787</v>
       </c>
       <c r="B147" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C147" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D147" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E147">
         <v>19</v>
@@ -12455,13 +12455,13 @@
         <v>6800</v>
       </c>
       <c r="B148" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C148" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D148" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E148">
         <v>12</v>
@@ -12535,13 +12535,13 @@
         <v>6878</v>
       </c>
       <c r="B149" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C149" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D149" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E149">
         <v>24</v>
@@ -12615,13 +12615,13 @@
         <v>6548</v>
       </c>
       <c r="B150" t="s">
+        <v>25</v>
+      </c>
+      <c r="C150" t="s">
         <v>26</v>
       </c>
-      <c r="C150" t="s">
-        <v>27</v>
-      </c>
       <c r="D150" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -12695,13 +12695,13 @@
         <v>6555</v>
       </c>
       <c r="B151" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C151" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D151" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -12775,13 +12775,13 @@
         <v>6805</v>
       </c>
       <c r="B152" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C152" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D152" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E152">
         <v>4</v>
@@ -12858,10 +12858,10 @@
         <v>15967961</v>
       </c>
       <c r="C153" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D153" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E153">
         <v>54</v>
@@ -12938,10 +12938,10 @@
         <v>12864933</v>
       </c>
       <c r="C154" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D154" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E154">
         <v>24</v>
@@ -13018,10 +13018,10 @@
         <v>15970137</v>
       </c>
       <c r="C155" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D155" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E155">
         <v>18</v>
@@ -13095,13 +13095,13 @@
         <v>6829</v>
       </c>
       <c r="B156" t="s">
+        <v>87</v>
+      </c>
+      <c r="C156" t="s">
+        <v>30</v>
+      </c>
+      <c r="D156" t="s">
         <v>88</v>
-      </c>
-      <c r="C156" t="s">
-        <v>31</v>
-      </c>
-      <c r="D156" t="s">
-        <v>89</v>
       </c>
       <c r="E156">
         <v>6</v>
@@ -13175,13 +13175,13 @@
         <v>6886</v>
       </c>
       <c r="B157" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C157" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D157" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E157">
         <v>2</v>
@@ -13255,13 +13255,13 @@
         <v>6890</v>
       </c>
       <c r="B158" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C158" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D158" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E158">
         <v>20</v>
@@ -13335,13 +13335,13 @@
         <v>6769</v>
       </c>
       <c r="B159" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C159" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D159" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E159">
         <v>15</v>
@@ -13415,13 +13415,13 @@
         <v>6880</v>
       </c>
       <c r="B160" t="s">
+        <v>91</v>
+      </c>
+      <c r="C160" t="s">
+        <v>30</v>
+      </c>
+      <c r="D160" t="s">
         <v>92</v>
-      </c>
-      <c r="C160" t="s">
-        <v>31</v>
-      </c>
-      <c r="D160" t="s">
-        <v>93</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -13495,13 +13495,13 @@
         <v>6881</v>
       </c>
       <c r="B161" t="s">
+        <v>93</v>
+      </c>
+      <c r="C161" t="s">
+        <v>30</v>
+      </c>
+      <c r="D161" t="s">
         <v>94</v>
-      </c>
-      <c r="C161" t="s">
-        <v>31</v>
-      </c>
-      <c r="D161" t="s">
-        <v>95</v>
       </c>
       <c r="E161">
         <v>10</v>
@@ -13575,13 +13575,13 @@
         <v>6952</v>
       </c>
       <c r="B162" t="s">
+        <v>29</v>
+      </c>
+      <c r="C162" t="s">
         <v>30</v>
       </c>
-      <c r="C162" t="s">
-        <v>31</v>
-      </c>
       <c r="D162" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E162">
         <v>28</v>
@@ -13655,13 +13655,13 @@
         <v>6815</v>
       </c>
       <c r="B163" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C163" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D163" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -13735,13 +13735,13 @@
         <v>6882</v>
       </c>
       <c r="B164" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C164" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D164" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -13818,10 +13818,10 @@
         <v>13828817</v>
       </c>
       <c r="C165" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D165" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E165">
         <v>12</v>
@@ -13898,10 +13898,10 @@
         <v>13832165</v>
       </c>
       <c r="C166" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D166" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E166">
         <v>12</v>
@@ -13975,13 +13975,13 @@
         <v>6806</v>
       </c>
       <c r="B167" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C167" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D167" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E167">
         <v>3</v>
@@ -14055,13 +14055,13 @@
         <v>6892</v>
       </c>
       <c r="B168" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C168" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D168" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E168">
         <v>15</v>
@@ -14135,13 +14135,13 @@
         <v>6816</v>
       </c>
       <c r="B169" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C169" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D169" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E169">
         <v>2</v>
@@ -14215,13 +14215,13 @@
         <v>6888</v>
       </c>
       <c r="B170" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C170" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D170" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E170">
         <v>34</v>
@@ -14295,13 +14295,13 @@
         <v>6808</v>
       </c>
       <c r="B171" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C171" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D171" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E171">
         <v>7</v>
@@ -14375,13 +14375,13 @@
         <v>6817</v>
       </c>
       <c r="B172" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C172" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D172" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E172">
         <v>2</v>
@@ -14455,13 +14455,13 @@
         <v>6879</v>
       </c>
       <c r="B173" t="s">
+        <v>31</v>
+      </c>
+      <c r="C173" t="s">
         <v>32</v>
       </c>
-      <c r="C173" t="s">
-        <v>33</v>
-      </c>
       <c r="D173" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E173">
         <v>4</v>
@@ -14535,13 +14535,13 @@
         <v>6807</v>
       </c>
       <c r="B174" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C174" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D174" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E174">
         <v>9</v>
@@ -14618,10 +14618,10 @@
         <v>13828817</v>
       </c>
       <c r="C175" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D175" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E175">
         <v>6</v>
@@ -14695,13 +14695,13 @@
         <v>6844</v>
       </c>
       <c r="B176" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C176" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D176" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E176">
         <v>16</v>
@@ -14775,13 +14775,13 @@
         <v>6845</v>
       </c>
       <c r="B177" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C177" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D177" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E177">
         <v>10</v>
@@ -14855,13 +14855,13 @@
         <v>6883</v>
       </c>
       <c r="B178" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C178" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D178" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E178">
         <v>20</v>
@@ -14935,13 +14935,13 @@
         <v>6884</v>
       </c>
       <c r="B179" t="s">
+        <v>106</v>
+      </c>
+      <c r="C179" t="s">
+        <v>30</v>
+      </c>
+      <c r="D179" t="s">
         <v>107</v>
-      </c>
-      <c r="C179" t="s">
-        <v>31</v>
-      </c>
-      <c r="D179" t="s">
-        <v>108</v>
       </c>
       <c r="E179">
         <v>6</v>
@@ -15015,13 +15015,13 @@
         <v>6891</v>
       </c>
       <c r="B180" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C180" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D180" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E180">
         <v>3</v>
@@ -15095,13 +15095,13 @@
         <v>6887</v>
       </c>
       <c r="B181" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C181" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D181" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E181">
         <v>10</v>
@@ -15175,13 +15175,13 @@
         <v>6949</v>
       </c>
       <c r="B182" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C182" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D182" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E182">
         <v>10</v>
@@ -15255,13 +15255,13 @@
         <v>6950</v>
       </c>
       <c r="B183" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C183" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D183" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E183">
         <v>9</v>
@@ -15335,13 +15335,13 @@
         <v>6951</v>
       </c>
       <c r="B184" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C184" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D184" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E184">
         <v>11</v>
@@ -15415,13 +15415,13 @@
         <v>6889</v>
       </c>
       <c r="B185" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C185" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D185" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E185">
         <v>4</v>

</xml_diff>

<commit_message>
fix: corrige leitura, cache e padronizacao da planilha PV no APS
</commit_message>
<xml_diff>
--- a/PV.xlsx
+++ b/PV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E24C35C0-F686-4EE9-99AF-7954304FC592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C1692E1-E65B-4B60-A4DE-CBD78A698E29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,9 +37,6 @@
     <t>DATA DE ENTREGA</t>
   </si>
   <si>
-    <t>CORTE - SERRA</t>
-  </si>
-  <si>
     <t>CORTE-PLASMA</t>
   </si>
   <si>
@@ -1192,7 +1189,10 @@
     <t>03/08/2026</t>
   </si>
   <si>
-    <t>QTE</t>
+    <t>QUANTIDADE</t>
+  </si>
+  <si>
+    <t>CORTE-SERRA</t>
   </si>
 </sst>
 </file>
@@ -1566,8 +1566,7 @@
     <col min="2" max="2" width="23.5546875" customWidth="1"/>
     <col min="3" max="3" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="17.21875" customWidth="1"/>
     <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.109375" bestFit="1" customWidth="1"/>
@@ -1603,81 +1602,81 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="H1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="M1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
         <v>39</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
         <v>40</v>
-      </c>
-      <c r="C2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D2" t="s">
-        <v>41</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1745,16 +1744,16 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" t="s">
-        <v>43</v>
-      </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -1822,16 +1821,16 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E4">
         <v>4</v>
@@ -1899,16 +1898,16 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s">
         <v>45</v>
       </c>
-      <c r="B5" t="s">
-        <v>46</v>
-      </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E5">
         <v>14</v>
@@ -1976,16 +1975,16 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
         <v>47</v>
-      </c>
-      <c r="B6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" t="s">
-        <v>48</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2053,16 +2052,16 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2130,16 +2129,16 @@
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
         <v>50</v>
       </c>
-      <c r="B8" t="s">
-        <v>51</v>
-      </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E8">
         <v>146</v>
@@ -2207,16 +2206,16 @@
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
         <v>55</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
         <v>56</v>
-      </c>
-      <c r="C9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" t="s">
-        <v>57</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2284,16 +2283,16 @@
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" t="s">
         <v>58</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" t="s">
         <v>59</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" t="s">
-        <v>60</v>
       </c>
       <c r="E10">
         <v>28</v>
@@ -2361,16 +2360,16 @@
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" t="s">
         <v>61</v>
       </c>
-      <c r="B11" t="s">
-        <v>62</v>
-      </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E11">
         <v>15</v>
@@ -2438,16 +2437,16 @@
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
         <v>63</v>
       </c>
-      <c r="B12" t="s">
-        <v>64</v>
-      </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E12">
         <v>2</v>
@@ -2515,16 +2514,16 @@
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" t="s">
         <v>65</v>
       </c>
-      <c r="B13" t="s">
-        <v>66</v>
-      </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E13">
         <v>4</v>
@@ -2592,16 +2591,16 @@
     </row>
     <row r="14" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" t="s">
         <v>67</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>68</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>69</v>
-      </c>
-      <c r="D14" t="s">
-        <v>70</v>
       </c>
       <c r="E14">
         <v>5</v>
@@ -2669,16 +2668,16 @@
     </row>
     <row r="15" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" t="s">
         <v>69</v>
-      </c>
-      <c r="D15" t="s">
-        <v>70</v>
       </c>
       <c r="E15">
         <v>5</v>
@@ -2746,16 +2745,16 @@
     </row>
     <row r="16" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" t="s">
         <v>69</v>
-      </c>
-      <c r="D16" t="s">
-        <v>70</v>
       </c>
       <c r="E16">
         <v>5</v>
@@ -2763,16 +2762,16 @@
     </row>
     <row r="17" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C17" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" t="s">
         <v>69</v>
-      </c>
-      <c r="D17" t="s">
-        <v>70</v>
       </c>
       <c r="E17">
         <v>5</v>
@@ -2840,16 +2839,16 @@
     </row>
     <row r="18" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
+        <v>68</v>
+      </c>
+      <c r="D18" t="s">
         <v>69</v>
-      </c>
-      <c r="D18" t="s">
-        <v>70</v>
       </c>
       <c r="E18">
         <v>5</v>
@@ -2917,16 +2916,16 @@
     </row>
     <row r="19" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C19" t="s">
+        <v>68</v>
+      </c>
+      <c r="D19" t="s">
         <v>69</v>
-      </c>
-      <c r="D19" t="s">
-        <v>70</v>
       </c>
       <c r="E19">
         <v>5</v>
@@ -2994,16 +2993,16 @@
     </row>
     <row r="20" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
+        <v>68</v>
+      </c>
+      <c r="D20" t="s">
         <v>69</v>
-      </c>
-      <c r="D20" t="s">
-        <v>70</v>
       </c>
       <c r="E20">
         <v>5</v>
@@ -3071,16 +3070,16 @@
     </row>
     <row r="21" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" t="s">
         <v>77</v>
       </c>
-      <c r="B21" t="s">
-        <v>78</v>
-      </c>
       <c r="C21" t="s">
+        <v>68</v>
+      </c>
+      <c r="D21" t="s">
         <v>69</v>
-      </c>
-      <c r="D21" t="s">
-        <v>70</v>
       </c>
       <c r="E21">
         <v>200</v>
@@ -3148,16 +3147,16 @@
     </row>
     <row r="22" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" t="s">
         <v>77</v>
       </c>
-      <c r="B22" t="s">
-        <v>78</v>
-      </c>
       <c r="C22" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" t="s">
         <v>69</v>
-      </c>
-      <c r="D22" t="s">
-        <v>70</v>
       </c>
       <c r="E22">
         <v>150</v>
@@ -3225,16 +3224,16 @@
     </row>
     <row r="23" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" t="s">
         <v>77</v>
       </c>
-      <c r="B23" t="s">
-        <v>78</v>
-      </c>
       <c r="C23" t="s">
+        <v>68</v>
+      </c>
+      <c r="D23" t="s">
         <v>69</v>
-      </c>
-      <c r="D23" t="s">
-        <v>70</v>
       </c>
       <c r="E23">
         <v>150</v>
@@ -3302,16 +3301,16 @@
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" t="s">
         <v>79</v>
       </c>
-      <c r="B24" t="s">
-        <v>80</v>
-      </c>
       <c r="C24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E24">
         <v>16</v>
@@ -3379,16 +3378,16 @@
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E25">
         <v>7</v>
@@ -3456,16 +3455,16 @@
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C26" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E26">
         <v>4</v>
@@ -3533,16 +3532,16 @@
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" t="s">
         <v>83</v>
       </c>
-      <c r="B27" t="s">
-        <v>84</v>
-      </c>
       <c r="C27" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D27" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -3610,16 +3609,16 @@
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B28" t="s">
         <v>85</v>
       </c>
-      <c r="B28" t="s">
-        <v>86</v>
-      </c>
       <c r="C28" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E28">
         <v>10</v>
@@ -3687,16 +3686,16 @@
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" t="s">
         <v>87</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
+        <v>24</v>
+      </c>
+      <c r="D29" t="s">
         <v>88</v>
-      </c>
-      <c r="C29" t="s">
-        <v>25</v>
-      </c>
-      <c r="D29" t="s">
-        <v>89</v>
       </c>
       <c r="E29">
         <v>7</v>
@@ -3764,16 +3763,16 @@
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C30" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D30" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -3841,16 +3840,16 @@
     </row>
     <row r="31" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" t="s">
         <v>92</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
+        <v>29</v>
+      </c>
+      <c r="D31" t="s">
         <v>93</v>
-      </c>
-      <c r="C31" t="s">
-        <v>30</v>
-      </c>
-      <c r="D31" t="s">
-        <v>94</v>
       </c>
       <c r="E31">
         <v>21</v>
@@ -3918,16 +3917,16 @@
     </row>
     <row r="32" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" t="s">
         <v>95</v>
       </c>
-      <c r="B32" t="s">
-        <v>96</v>
-      </c>
       <c r="C32" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D32" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E32">
         <v>24</v>
@@ -3995,16 +3994,16 @@
     </row>
     <row r="33" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" t="s">
         <v>97</v>
       </c>
-      <c r="B33" t="s">
-        <v>98</v>
-      </c>
       <c r="C33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D33" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E33">
         <v>12</v>
@@ -4072,16 +4071,16 @@
     </row>
     <row r="34" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B34" t="s">
         <v>99</v>
       </c>
-      <c r="B34" t="s">
-        <v>100</v>
-      </c>
       <c r="C34" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D34" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E34">
         <v>12</v>
@@ -4149,16 +4148,16 @@
     </row>
     <row r="35" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35" t="s">
         <v>101</v>
       </c>
-      <c r="B35" t="s">
-        <v>102</v>
-      </c>
       <c r="C35" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D35" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E35">
         <v>12</v>
@@ -4226,16 +4225,16 @@
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B36" t="s">
         <v>103</v>
       </c>
-      <c r="B36" t="s">
-        <v>104</v>
-      </c>
       <c r="C36" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D36" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E36">
         <v>6</v>
@@ -4303,16 +4302,16 @@
     </row>
     <row r="37" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37" t="s">
         <v>29</v>
       </c>
-      <c r="C37" t="s">
-        <v>30</v>
-      </c>
       <c r="D37" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E37">
         <v>27</v>
@@ -4380,16 +4379,16 @@
     </row>
     <row r="38" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B38" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C38" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D38" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E38">
         <v>54</v>
@@ -4457,16 +4456,16 @@
     </row>
     <row r="39" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B39" t="s">
         <v>107</v>
       </c>
-      <c r="B39" t="s">
-        <v>108</v>
-      </c>
       <c r="C39" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E39">
         <v>54</v>
@@ -4534,16 +4533,16 @@
     </row>
     <row r="40" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B40" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C40" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D40" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E40">
         <v>27</v>
@@ -4611,16 +4610,16 @@
     </row>
     <row r="41" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B41" t="s">
         <v>110</v>
       </c>
-      <c r="B41" t="s">
-        <v>111</v>
-      </c>
       <c r="C41" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D41" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E41">
         <v>27</v>
@@ -4688,16 +4687,16 @@
     </row>
     <row r="42" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B42" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C42" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D42" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E42">
         <v>27</v>
@@ -4765,16 +4764,16 @@
     </row>
     <row r="43" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B43" t="s">
         <v>113</v>
       </c>
-      <c r="B43" t="s">
-        <v>114</v>
-      </c>
       <c r="C43" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D43" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E43">
         <v>54</v>
@@ -4842,16 +4841,16 @@
     </row>
     <row r="44" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B44" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C44" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D44" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E44">
         <v>100</v>
@@ -4919,16 +4918,16 @@
     </row>
     <row r="45" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B45" t="s">
         <v>116</v>
       </c>
-      <c r="B45" t="s">
-        <v>117</v>
-      </c>
       <c r="C45" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D45" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E45">
         <v>48</v>
@@ -4996,16 +4995,16 @@
     </row>
     <row r="46" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B46" t="s">
         <v>118</v>
       </c>
-      <c r="B46" t="s">
-        <v>119</v>
-      </c>
       <c r="C46" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D46" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E46">
         <v>24</v>
@@ -5073,16 +5072,16 @@
     </row>
     <row r="47" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B47" t="s">
         <v>120</v>
       </c>
-      <c r="B47" t="s">
-        <v>121</v>
-      </c>
       <c r="C47" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D47" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E47">
         <v>3</v>
@@ -5150,16 +5149,16 @@
     </row>
     <row r="48" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B48" t="s">
         <v>122</v>
       </c>
-      <c r="B48" t="s">
-        <v>123</v>
-      </c>
       <c r="C48" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D48" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E48">
         <v>12</v>
@@ -5227,16 +5226,16 @@
     </row>
     <row r="49" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B49" t="s">
         <v>124</v>
       </c>
-      <c r="B49" t="s">
-        <v>125</v>
-      </c>
       <c r="C49" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D49" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E49">
         <v>6</v>
@@ -5304,16 +5303,16 @@
     </row>
     <row r="50" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B50" t="s">
         <v>126</v>
       </c>
-      <c r="B50" t="s">
-        <v>127</v>
-      </c>
       <c r="C50" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D50" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E50">
         <v>6</v>
@@ -5381,16 +5380,16 @@
     </row>
     <row r="51" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B51" t="s">
         <v>128</v>
       </c>
-      <c r="B51" t="s">
-        <v>129</v>
-      </c>
       <c r="C51" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D51" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E51">
         <v>6</v>
@@ -5458,16 +5457,16 @@
     </row>
     <row r="52" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B52" t="s">
         <v>130</v>
       </c>
-      <c r="B52" t="s">
-        <v>131</v>
-      </c>
       <c r="C52" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D52" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E52">
         <v>6</v>
@@ -5535,16 +5534,16 @@
     </row>
     <row r="53" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B53" t="s">
         <v>132</v>
       </c>
-      <c r="B53" t="s">
-        <v>133</v>
-      </c>
       <c r="C53" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D53" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E53">
         <v>6</v>
@@ -5612,16 +5611,16 @@
     </row>
     <row r="54" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B54" t="s">
         <v>134</v>
       </c>
-      <c r="B54" t="s">
-        <v>135</v>
-      </c>
       <c r="C54" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D54" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E54">
         <v>3</v>
@@ -5689,16 +5688,16 @@
     </row>
     <row r="55" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B55" t="s">
         <v>136</v>
       </c>
-      <c r="B55" t="s">
-        <v>137</v>
-      </c>
       <c r="C55" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D55" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E55">
         <v>3</v>
@@ -5766,16 +5765,16 @@
     </row>
     <row r="56" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B56" t="s">
         <v>138</v>
       </c>
-      <c r="B56" t="s">
-        <v>139</v>
-      </c>
       <c r="C56" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D56" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E56">
         <v>6</v>
@@ -5843,16 +5842,16 @@
     </row>
     <row r="57" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B57" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C57" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D57" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E57">
         <v>100</v>
@@ -5920,16 +5919,16 @@
     </row>
     <row r="58" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B58" t="s">
         <v>141</v>
       </c>
-      <c r="B58" t="s">
-        <v>142</v>
-      </c>
       <c r="C58" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D58" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E58">
         <v>6</v>
@@ -5997,16 +5996,16 @@
     </row>
     <row r="59" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B59" t="s">
         <v>143</v>
       </c>
-      <c r="B59" t="s">
-        <v>144</v>
-      </c>
       <c r="C59" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D59" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E59">
         <v>6</v>
@@ -6074,16 +6073,16 @@
     </row>
     <row r="60" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B60" t="s">
         <v>145</v>
       </c>
-      <c r="B60" t="s">
-        <v>146</v>
-      </c>
       <c r="C60" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D60" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E60">
         <v>6</v>
@@ -6151,16 +6150,16 @@
     </row>
     <row r="61" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B61" t="s">
         <v>147</v>
       </c>
-      <c r="B61" t="s">
-        <v>148</v>
-      </c>
       <c r="C61" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D61" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E61">
         <v>6</v>
@@ -6228,16 +6227,16 @@
     </row>
     <row r="62" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B62" t="s">
         <v>149</v>
       </c>
-      <c r="B62" t="s">
-        <v>150</v>
-      </c>
       <c r="C62" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D62" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E62">
         <v>6</v>
@@ -6305,16 +6304,16 @@
     </row>
     <row r="63" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B63" t="s">
         <v>151</v>
       </c>
-      <c r="B63" t="s">
-        <v>152</v>
-      </c>
       <c r="C63" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D63" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E63">
         <v>6</v>
@@ -6382,16 +6381,16 @@
     </row>
     <row r="64" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B64" t="s">
         <v>153</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
+        <v>24</v>
+      </c>
+      <c r="D64" t="s">
         <v>154</v>
-      </c>
-      <c r="C64" t="s">
-        <v>25</v>
-      </c>
-      <c r="D64" t="s">
-        <v>155</v>
       </c>
       <c r="E64">
         <v>62</v>
@@ -6459,16 +6458,16 @@
     </row>
     <row r="65" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B65" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C65" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D65" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -6536,16 +6535,16 @@
     </row>
     <row r="66" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B66" t="s">
+        <v>23</v>
+      </c>
+      <c r="C66" t="s">
         <v>24</v>
       </c>
-      <c r="C66" t="s">
-        <v>25</v>
-      </c>
       <c r="D66" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E66">
         <v>51</v>
@@ -6613,16 +6612,16 @@
     </row>
     <row r="67" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B67" t="s">
         <v>158</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C67" t="s">
         <v>159</v>
       </c>
-      <c r="C67" t="s">
-        <v>160</v>
-      </c>
       <c r="D67" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E67">
         <v>1</v>
@@ -6630,16 +6629,16 @@
     </row>
     <row r="68" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B68" t="s">
         <v>161</v>
       </c>
-      <c r="B68" t="s">
-        <v>162</v>
-      </c>
       <c r="C68" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D68" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E68">
         <v>5</v>
@@ -6707,16 +6706,16 @@
     </row>
     <row r="69" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B69" t="s">
+        <v>39</v>
+      </c>
+      <c r="C69" t="s">
+        <v>24</v>
+      </c>
+      <c r="D69" t="s">
         <v>163</v>
-      </c>
-      <c r="B69" t="s">
-        <v>40</v>
-      </c>
-      <c r="C69" t="s">
-        <v>25</v>
-      </c>
-      <c r="D69" t="s">
-        <v>164</v>
       </c>
       <c r="E69">
         <v>1</v>
@@ -6784,16 +6783,16 @@
     </row>
     <row r="70" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B70" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C70" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D70" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E70">
         <v>1</v>
@@ -6861,16 +6860,16 @@
     </row>
     <row r="71" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B71" t="s">
         <v>166</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
+        <v>24</v>
+      </c>
+      <c r="D71" t="s">
         <v>167</v>
-      </c>
-      <c r="C71" t="s">
-        <v>25</v>
-      </c>
-      <c r="D71" t="s">
-        <v>168</v>
       </c>
       <c r="E71">
         <v>3</v>
@@ -6938,16 +6937,16 @@
     </row>
     <row r="72" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B72" t="s">
+        <v>92</v>
+      </c>
+      <c r="C72" t="s">
+        <v>29</v>
+      </c>
+      <c r="D72" t="s">
         <v>169</v>
-      </c>
-      <c r="B72" t="s">
-        <v>93</v>
-      </c>
-      <c r="C72" t="s">
-        <v>30</v>
-      </c>
-      <c r="D72" t="s">
-        <v>170</v>
       </c>
       <c r="E72">
         <v>24</v>
@@ -7015,16 +7014,16 @@
     </row>
     <row r="73" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B73" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C73" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D73" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E73">
         <v>123</v>
@@ -7092,16 +7091,16 @@
     </row>
     <row r="74" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B74" t="s">
         <v>172</v>
       </c>
-      <c r="B74" t="s">
-        <v>173</v>
-      </c>
       <c r="C74" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D74" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E74">
         <v>8</v>
@@ -7169,16 +7168,16 @@
     </row>
     <row r="75" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B75" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C75" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D75" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E75">
         <v>4</v>
@@ -7246,16 +7245,16 @@
     </row>
     <row r="76" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B76" t="s">
         <v>175</v>
       </c>
-      <c r="B76" t="s">
-        <v>176</v>
-      </c>
       <c r="C76" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D76" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E76">
         <v>3</v>
@@ -7323,16 +7322,16 @@
     </row>
     <row r="77" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B77" t="s">
         <v>177</v>
       </c>
-      <c r="B77" t="s">
-        <v>178</v>
-      </c>
       <c r="C77" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D77" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E77">
         <v>6</v>
@@ -7400,16 +7399,16 @@
     </row>
     <row r="78" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B78" t="s">
         <v>179</v>
       </c>
-      <c r="B78" t="s">
-        <v>180</v>
-      </c>
       <c r="C78" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D78" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E78">
         <v>9</v>
@@ -7477,16 +7476,16 @@
     </row>
     <row r="79" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B79" t="s">
         <v>181</v>
       </c>
-      <c r="B79" t="s">
-        <v>182</v>
-      </c>
       <c r="C79" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D79" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E79">
         <v>9</v>
@@ -7554,16 +7553,16 @@
     </row>
     <row r="80" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B80" t="s">
         <v>183</v>
       </c>
-      <c r="B80" t="s">
-        <v>184</v>
-      </c>
       <c r="C80" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D80" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E80">
         <v>9</v>
@@ -7631,16 +7630,16 @@
     </row>
     <row r="81" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B81" t="s">
         <v>185</v>
       </c>
-      <c r="B81" t="s">
-        <v>186</v>
-      </c>
       <c r="C81" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D81" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E81">
         <v>36</v>
@@ -7708,16 +7707,16 @@
     </row>
     <row r="82" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B82" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C82" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D82" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E82">
         <v>9</v>
@@ -7785,16 +7784,16 @@
     </row>
     <row r="83" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B83" t="s">
         <v>188</v>
       </c>
-      <c r="B83" t="s">
-        <v>189</v>
-      </c>
       <c r="C83" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D83" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E83">
         <v>10</v>
@@ -7862,16 +7861,16 @@
     </row>
     <row r="84" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B84" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C84" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D84" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E84">
         <v>20</v>
@@ -7939,16 +7938,16 @@
     </row>
     <row r="85" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B85" t="s">
         <v>191</v>
       </c>
-      <c r="B85" t="s">
-        <v>192</v>
-      </c>
       <c r="C85" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D85" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E85">
         <v>6</v>
@@ -8016,16 +8015,16 @@
     </row>
     <row r="86" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B86" t="s">
         <v>193</v>
       </c>
-      <c r="B86" t="s">
-        <v>194</v>
-      </c>
       <c r="C86" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D86" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E86">
         <v>3</v>
@@ -8093,16 +8092,16 @@
     </row>
     <row r="87" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B87" t="s">
         <v>195</v>
       </c>
-      <c r="B87" t="s">
-        <v>196</v>
-      </c>
       <c r="C87" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D87" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E87">
         <v>6</v>
@@ -8170,16 +8169,16 @@
     </row>
     <row r="88" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B88" t="s">
         <v>197</v>
       </c>
-      <c r="B88" t="s">
-        <v>198</v>
-      </c>
       <c r="C88" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D88" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E88">
         <v>6</v>
@@ -8247,16 +8246,16 @@
     </row>
     <row r="89" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B89" t="s">
         <v>199</v>
       </c>
-      <c r="B89" t="s">
-        <v>200</v>
-      </c>
       <c r="C89" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D89" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E89">
         <v>3</v>
@@ -8324,16 +8323,16 @@
     </row>
     <row r="90" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B90" t="s">
         <v>201</v>
       </c>
-      <c r="B90" t="s">
-        <v>202</v>
-      </c>
       <c r="C90" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D90" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E90">
         <v>6</v>
@@ -8401,16 +8400,16 @@
     </row>
     <row r="91" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B91" t="s">
         <v>203</v>
       </c>
-      <c r="B91" t="s">
-        <v>204</v>
-      </c>
       <c r="C91" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D91" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E91">
         <v>12</v>
@@ -8478,16 +8477,16 @@
     </row>
     <row r="92" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B92" t="s">
         <v>205</v>
       </c>
-      <c r="B92" t="s">
-        <v>206</v>
-      </c>
       <c r="C92" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D92" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E92">
         <v>6</v>
@@ -8555,16 +8554,16 @@
     </row>
     <row r="93" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B93" t="s">
         <v>207</v>
       </c>
-      <c r="B93" t="s">
-        <v>208</v>
-      </c>
       <c r="C93" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D93" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E93">
         <v>6</v>
@@ -8632,16 +8631,16 @@
     </row>
     <row r="94" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B94" t="s">
         <v>209</v>
       </c>
-      <c r="B94" t="s">
-        <v>210</v>
-      </c>
       <c r="C94" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D94" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E94">
         <v>6</v>
@@ -8709,16 +8708,16 @@
     </row>
     <row r="95" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B95" t="s">
         <v>211</v>
       </c>
-      <c r="B95" t="s">
+      <c r="C95" t="s">
+        <v>24</v>
+      </c>
+      <c r="D95" t="s">
         <v>212</v>
-      </c>
-      <c r="C95" t="s">
-        <v>25</v>
-      </c>
-      <c r="D95" t="s">
-        <v>213</v>
       </c>
       <c r="E95">
         <v>2</v>
@@ -8786,16 +8785,16 @@
     </row>
     <row r="96" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B96" t="s">
+        <v>166</v>
+      </c>
+      <c r="C96" t="s">
+        <v>24</v>
+      </c>
+      <c r="D96" t="s">
         <v>214</v>
-      </c>
-      <c r="B96" t="s">
-        <v>167</v>
-      </c>
-      <c r="C96" t="s">
-        <v>25</v>
-      </c>
-      <c r="D96" t="s">
-        <v>215</v>
       </c>
       <c r="E96">
         <v>3</v>
@@ -8863,16 +8862,16 @@
     </row>
     <row r="97" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B97" t="s">
         <v>216</v>
       </c>
-      <c r="B97" t="s">
+      <c r="C97" t="s">
+        <v>24</v>
+      </c>
+      <c r="D97" t="s">
         <v>217</v>
-      </c>
-      <c r="C97" t="s">
-        <v>25</v>
-      </c>
-      <c r="D97" t="s">
-        <v>218</v>
       </c>
       <c r="E97">
         <v>10</v>
@@ -8940,16 +8939,16 @@
     </row>
     <row r="98" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B98" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C98" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D98" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E98">
         <v>7</v>
@@ -9017,16 +9016,16 @@
     </row>
     <row r="99" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B99" t="s">
         <v>220</v>
       </c>
-      <c r="B99" t="s">
-        <v>221</v>
-      </c>
       <c r="C99" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D99" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E99">
         <v>200</v>
@@ -9094,16 +9093,16 @@
     </row>
     <row r="100" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B100" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C100" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D100" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -9171,16 +9170,16 @@
     </row>
     <row r="101" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B101" t="s">
         <v>223</v>
       </c>
-      <c r="B101" t="s">
+      <c r="C101" t="s">
+        <v>24</v>
+      </c>
+      <c r="D101" t="s">
         <v>224</v>
-      </c>
-      <c r="C101" t="s">
-        <v>25</v>
-      </c>
-      <c r="D101" t="s">
-        <v>225</v>
       </c>
       <c r="E101">
         <v>32</v>
@@ -9248,16 +9247,16 @@
     </row>
     <row r="102" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B102" t="s">
         <v>226</v>
       </c>
-      <c r="B102" t="s">
+      <c r="C102" t="s">
         <v>227</v>
       </c>
-      <c r="C102" t="s">
+      <c r="D102" t="s">
         <v>228</v>
-      </c>
-      <c r="D102" t="s">
-        <v>229</v>
       </c>
       <c r="E102">
         <v>48</v>
@@ -9325,16 +9324,16 @@
     </row>
     <row r="103" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B103" t="s">
         <v>230</v>
       </c>
-      <c r="B103" t="s">
-        <v>231</v>
-      </c>
       <c r="C103" t="s">
+        <v>227</v>
+      </c>
+      <c r="D103" t="s">
         <v>228</v>
-      </c>
-      <c r="D103" t="s">
-        <v>229</v>
       </c>
       <c r="E103">
         <v>48</v>
@@ -9402,16 +9401,16 @@
     </row>
     <row r="104" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B104" t="s">
         <v>232</v>
       </c>
-      <c r="B104" t="s">
+      <c r="C104" t="s">
+        <v>24</v>
+      </c>
+      <c r="D104" t="s">
         <v>233</v>
-      </c>
-      <c r="C104" t="s">
-        <v>25</v>
-      </c>
-      <c r="D104" t="s">
-        <v>234</v>
       </c>
       <c r="E104">
         <v>5</v>
@@ -9479,16 +9478,16 @@
     </row>
     <row r="105" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B105" t="s">
         <v>235</v>
       </c>
-      <c r="B105" t="s">
-        <v>236</v>
-      </c>
       <c r="C105" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D105" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E105">
         <v>18</v>
@@ -9556,16 +9555,16 @@
     </row>
     <row r="106" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B106" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C106" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D106" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E106">
         <v>50</v>
@@ -9633,16 +9632,16 @@
     </row>
     <row r="107" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B107" t="s">
         <v>238</v>
       </c>
-      <c r="B107" t="s">
-        <v>239</v>
-      </c>
       <c r="C107" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D107" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E107">
         <v>6</v>
@@ -9710,16 +9709,16 @@
     </row>
     <row r="108" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B108" t="s">
         <v>240</v>
       </c>
-      <c r="B108" t="s">
-        <v>241</v>
-      </c>
       <c r="C108" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D108" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E108">
         <v>12</v>
@@ -9787,16 +9786,16 @@
     </row>
     <row r="109" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B109" t="s">
         <v>242</v>
       </c>
-      <c r="B109" t="s">
-        <v>243</v>
-      </c>
       <c r="C109" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D109" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E109">
         <v>6</v>
@@ -9864,16 +9863,16 @@
     </row>
     <row r="110" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B110" t="s">
         <v>244</v>
       </c>
-      <c r="B110" t="s">
-        <v>245</v>
-      </c>
       <c r="C110" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D110" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E110">
         <v>6</v>
@@ -9941,16 +9940,16 @@
     </row>
     <row r="111" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B111" t="s">
         <v>246</v>
       </c>
-      <c r="B111" t="s">
-        <v>247</v>
-      </c>
       <c r="C111" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D111" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E111">
         <v>6</v>
@@ -10018,16 +10017,16 @@
     </row>
     <row r="112" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B112" t="s">
         <v>248</v>
       </c>
-      <c r="B112" t="s">
-        <v>249</v>
-      </c>
       <c r="C112" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D112" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E112">
         <v>6</v>
@@ -10095,16 +10094,16 @@
     </row>
     <row r="113" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B113" t="s">
         <v>250</v>
       </c>
-      <c r="B113" t="s">
-        <v>251</v>
-      </c>
       <c r="C113" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D113" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E113">
         <v>6</v>
@@ -10172,16 +10171,16 @@
     </row>
     <row r="114" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B114" t="s">
+        <v>79</v>
+      </c>
+      <c r="C114" t="s">
+        <v>24</v>
+      </c>
+      <c r="D114" t="s">
         <v>252</v>
-      </c>
-      <c r="B114" t="s">
-        <v>80</v>
-      </c>
-      <c r="C114" t="s">
-        <v>25</v>
-      </c>
-      <c r="D114" t="s">
-        <v>253</v>
       </c>
       <c r="E114">
         <v>6</v>
@@ -10249,16 +10248,16 @@
     </row>
     <row r="115" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B115" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C115" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D115" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E115">
         <v>3</v>
@@ -10326,16 +10325,16 @@
     </row>
     <row r="116" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B116" t="s">
         <v>255</v>
       </c>
-      <c r="B116" t="s">
-        <v>256</v>
-      </c>
       <c r="C116" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D116" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E116">
         <v>50</v>
@@ -10403,16 +10402,16 @@
     </row>
     <row r="117" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B117" t="s">
         <v>257</v>
       </c>
-      <c r="B117" t="s">
+      <c r="C117" t="s">
+        <v>24</v>
+      </c>
+      <c r="D117" t="s">
         <v>258</v>
-      </c>
-      <c r="C117" t="s">
-        <v>25</v>
-      </c>
-      <c r="D117" t="s">
-        <v>259</v>
       </c>
       <c r="E117">
         <v>9</v>
@@ -10480,16 +10479,16 @@
     </row>
     <row r="118" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B118" t="s">
         <v>260</v>
       </c>
-      <c r="B118" t="s">
+      <c r="C118" t="s">
+        <v>29</v>
+      </c>
+      <c r="D118" t="s">
         <v>261</v>
-      </c>
-      <c r="C118" t="s">
-        <v>30</v>
-      </c>
-      <c r="D118" t="s">
-        <v>262</v>
       </c>
       <c r="E118">
         <v>39</v>
@@ -10557,16 +10556,16 @@
     </row>
     <row r="119" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B119" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C119" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D119" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E119">
         <v>18</v>
@@ -10634,16 +10633,16 @@
     </row>
     <row r="120" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B120" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C120" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D120" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E120">
         <v>18</v>
@@ -10711,16 +10710,16 @@
     </row>
     <row r="121" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B121" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C121" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D121" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E121">
         <v>72</v>
@@ -10788,16 +10787,16 @@
     </row>
     <row r="122" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B122" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C122" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D122" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E122">
         <v>15</v>
@@ -10865,16 +10864,16 @@
     </row>
     <row r="123" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B123" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C123" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D123" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E123">
         <v>15</v>
@@ -10942,16 +10941,16 @@
     </row>
     <row r="124" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B124" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C124" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D124" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E124">
         <v>50</v>
@@ -11019,16 +11018,16 @@
     </row>
     <row r="125" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B125" t="s">
         <v>269</v>
       </c>
-      <c r="B125" t="s">
-        <v>270</v>
-      </c>
       <c r="C125" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D125" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E125">
         <v>60</v>
@@ -11096,16 +11095,16 @@
     </row>
     <row r="126" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B126" t="s">
         <v>271</v>
       </c>
-      <c r="B126" t="s">
-        <v>272</v>
-      </c>
       <c r="C126" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D126" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E126">
         <v>21</v>
@@ -11173,16 +11172,16 @@
     </row>
     <row r="127" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B127" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C127" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D127" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E127">
         <v>27</v>
@@ -11250,16 +11249,16 @@
     </row>
     <row r="128" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B128" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C128" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D128" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E128">
         <v>624</v>
@@ -11327,16 +11326,16 @@
     </row>
     <row r="129" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B129" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C129" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D129" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E129">
         <v>21</v>
@@ -11404,16 +11403,16 @@
     </row>
     <row r="130" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B130" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C130" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D130" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E130">
         <v>57</v>
@@ -11481,16 +11480,16 @@
     </row>
     <row r="131" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B131" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C131" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D131" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E131">
         <v>6</v>
@@ -11558,16 +11557,16 @@
     </row>
     <row r="132" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B132" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C132" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D132" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E132">
         <v>18</v>
@@ -11635,16 +11634,16 @@
     </row>
     <row r="133" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B133" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C133" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D133" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E133">
         <v>15</v>
@@ -11712,16 +11711,16 @@
     </row>
     <row r="134" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B134" t="s">
         <v>280</v>
       </c>
-      <c r="B134" t="s">
-        <v>281</v>
-      </c>
       <c r="C134" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D134" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E134">
         <v>78</v>
@@ -11789,16 +11788,16 @@
     </row>
     <row r="135" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B135" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C135" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D135" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E135">
         <v>3</v>
@@ -11866,16 +11865,16 @@
     </row>
     <row r="136" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B136" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C136" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D136" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E136">
         <v>33</v>
@@ -11943,16 +11942,16 @@
     </row>
     <row r="137" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B137" t="s">
         <v>284</v>
       </c>
-      <c r="B137" t="s">
-        <v>285</v>
-      </c>
       <c r="C137" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D137" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E137">
         <v>6</v>
@@ -12020,16 +12019,16 @@
     </row>
     <row r="138" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B138" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C138" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D138" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E138">
         <v>21</v>
@@ -12097,16 +12096,16 @@
     </row>
     <row r="139" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B139" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C139" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D139" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E139">
         <v>6</v>
@@ -12174,16 +12173,16 @@
     </row>
     <row r="140" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B140" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C140" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D140" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E140">
         <v>6</v>
@@ -12251,16 +12250,16 @@
     </row>
     <row r="141" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B141" t="s">
         <v>289</v>
       </c>
-      <c r="B141" t="s">
-        <v>290</v>
-      </c>
       <c r="C141" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D141" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E141">
         <v>6</v>
@@ -12328,16 +12327,16 @@
     </row>
     <row r="142" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B142" t="s">
         <v>291</v>
       </c>
-      <c r="B142" t="s">
-        <v>292</v>
-      </c>
       <c r="C142" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D142" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E142">
         <v>10</v>
@@ -12405,16 +12404,16 @@
     </row>
     <row r="143" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B143" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C143" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D143" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E143">
         <v>15</v>
@@ -12482,16 +12481,16 @@
     </row>
     <row r="144" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B144" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C144" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D144" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E144">
         <v>30</v>
@@ -12559,16 +12558,16 @@
     </row>
     <row r="145" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B145" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C145" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D145" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E145">
         <v>15</v>
@@ -12636,16 +12635,16 @@
     </row>
     <row r="146" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B146" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C146" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D146" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E146">
         <v>15</v>
@@ -12713,16 +12712,16 @@
     </row>
     <row r="147" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B147" t="s">
         <v>297</v>
       </c>
-      <c r="B147" t="s">
-        <v>298</v>
-      </c>
       <c r="C147" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D147" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E147">
         <v>9</v>
@@ -12790,16 +12789,16 @@
     </row>
     <row r="148" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B148" t="s">
         <v>299</v>
       </c>
-      <c r="B148" t="s">
-        <v>300</v>
-      </c>
       <c r="C148" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D148" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E148">
         <v>9</v>
@@ -12867,16 +12866,16 @@
     </row>
     <row r="149" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B149" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C149" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D149" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E149">
         <v>9</v>
@@ -12944,16 +12943,16 @@
     </row>
     <row r="150" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B150" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C150" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D150" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E150">
         <v>6</v>
@@ -13021,16 +13020,16 @@
     </row>
     <row r="151" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B151" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C151" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D151" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E151">
         <v>6</v>
@@ -13098,16 +13097,16 @@
     </row>
     <row r="152" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B152" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C152" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D152" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E152">
         <v>3</v>
@@ -13175,16 +13174,16 @@
     </row>
     <row r="153" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B153" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C153" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D153" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E153">
         <v>3</v>
@@ -13252,16 +13251,16 @@
     </row>
     <row r="154" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B154" t="s">
+        <v>28</v>
+      </c>
+      <c r="C154" t="s">
         <v>29</v>
       </c>
-      <c r="C154" t="s">
-        <v>30</v>
-      </c>
       <c r="D154" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E154">
         <v>21</v>
@@ -13329,16 +13328,16 @@
     </row>
     <row r="155" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B155" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C155" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D155" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E155">
         <v>42</v>
@@ -13406,16 +13405,16 @@
     </row>
     <row r="156" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B156" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C156" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D156" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E156">
         <v>42</v>
@@ -13483,16 +13482,16 @@
     </row>
     <row r="157" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B157" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C157" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D157" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E157">
         <v>21</v>
@@ -13560,16 +13559,16 @@
     </row>
     <row r="158" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B158" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C158" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D158" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E158">
         <v>21</v>
@@ -13637,16 +13636,16 @@
     </row>
     <row r="159" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B159" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C159" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D159" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E159">
         <v>21</v>
@@ -13714,16 +13713,16 @@
     </row>
     <row r="160" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B160" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C160" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D160" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E160">
         <v>42</v>
@@ -13791,16 +13790,16 @@
     </row>
     <row r="161" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="B161" t="s">
+        <v>211</v>
+      </c>
+      <c r="C161" t="s">
+        <v>24</v>
+      </c>
+      <c r="D161" t="s">
         <v>313</v>
-      </c>
-      <c r="B161" t="s">
-        <v>212</v>
-      </c>
-      <c r="C161" t="s">
-        <v>25</v>
-      </c>
-      <c r="D161" t="s">
-        <v>314</v>
       </c>
       <c r="E161">
         <v>19</v>
@@ -13868,16 +13867,16 @@
     </row>
     <row r="162" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B162" t="s">
+        <v>83</v>
+      </c>
+      <c r="C162" t="s">
+        <v>24</v>
+      </c>
+      <c r="D162" t="s">
         <v>315</v>
-      </c>
-      <c r="B162" t="s">
-        <v>84</v>
-      </c>
-      <c r="C162" t="s">
-        <v>25</v>
-      </c>
-      <c r="D162" t="s">
-        <v>316</v>
       </c>
       <c r="E162">
         <v>12</v>
@@ -13945,16 +13944,16 @@
     </row>
     <row r="163" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="B163" t="s">
         <v>317</v>
       </c>
-      <c r="B163" t="s">
-        <v>318</v>
-      </c>
       <c r="C163" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D163" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E163">
         <v>24</v>
@@ -14022,16 +14021,16 @@
     </row>
     <row r="164" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B164" t="s">
+        <v>39</v>
+      </c>
+      <c r="C164" t="s">
+        <v>24</v>
+      </c>
+      <c r="D164" t="s">
         <v>319</v>
-      </c>
-      <c r="B164" t="s">
-        <v>40</v>
-      </c>
-      <c r="C164" t="s">
-        <v>25</v>
-      </c>
-      <c r="D164" t="s">
-        <v>320</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -14099,16 +14098,16 @@
     </row>
     <row r="165" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B165" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C165" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D165" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E165">
         <v>1</v>
@@ -14176,16 +14175,16 @@
     </row>
     <row r="166" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B166" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C166" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D166" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E166">
         <v>4</v>
@@ -14253,16 +14252,16 @@
     </row>
     <row r="167" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B167" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C167" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D167" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E167">
         <v>24</v>
@@ -14330,16 +14329,16 @@
     </row>
     <row r="168" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B168" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C168" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D168" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E168">
         <v>54</v>
@@ -14407,16 +14406,16 @@
     </row>
     <row r="169" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B169" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C169" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D169" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E169">
         <v>18</v>
@@ -14484,16 +14483,16 @@
     </row>
     <row r="170" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="B170" t="s">
         <v>326</v>
       </c>
-      <c r="B170" t="s">
+      <c r="C170" t="s">
+        <v>24</v>
+      </c>
+      <c r="D170" t="s">
         <v>327</v>
-      </c>
-      <c r="C170" t="s">
-        <v>25</v>
-      </c>
-      <c r="D170" t="s">
-        <v>328</v>
       </c>
       <c r="E170">
         <v>6</v>
@@ -14561,16 +14560,16 @@
     </row>
     <row r="171" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B171" t="s">
+        <v>172</v>
+      </c>
+      <c r="C171" t="s">
+        <v>24</v>
+      </c>
+      <c r="D171" t="s">
         <v>329</v>
-      </c>
-      <c r="B171" t="s">
-        <v>173</v>
-      </c>
-      <c r="C171" t="s">
-        <v>25</v>
-      </c>
-      <c r="D171" t="s">
-        <v>330</v>
       </c>
       <c r="E171">
         <v>20</v>
@@ -14638,16 +14637,16 @@
     </row>
     <row r="172" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B172" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C172" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D172" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E172">
         <v>2</v>
@@ -14715,16 +14714,16 @@
     </row>
     <row r="173" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="B173" t="s">
+        <v>79</v>
+      </c>
+      <c r="C173" t="s">
+        <v>24</v>
+      </c>
+      <c r="D173" t="s">
         <v>332</v>
-      </c>
-      <c r="B173" t="s">
-        <v>80</v>
-      </c>
-      <c r="C173" t="s">
-        <v>25</v>
-      </c>
-      <c r="D173" t="s">
-        <v>333</v>
       </c>
       <c r="E173">
         <v>15</v>
@@ -14792,16 +14791,16 @@
     </row>
     <row r="174" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B174" t="s">
         <v>334</v>
       </c>
-      <c r="B174" t="s">
+      <c r="C174" t="s">
+        <v>24</v>
+      </c>
+      <c r="D174" t="s">
         <v>335</v>
-      </c>
-      <c r="C174" t="s">
-        <v>25</v>
-      </c>
-      <c r="D174" t="s">
-        <v>336</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -14869,16 +14868,16 @@
     </row>
     <row r="175" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B175" t="s">
         <v>337</v>
       </c>
-      <c r="B175" t="s">
+      <c r="C175" t="s">
+        <v>24</v>
+      </c>
+      <c r="D175" t="s">
         <v>338</v>
-      </c>
-      <c r="C175" t="s">
-        <v>25</v>
-      </c>
-      <c r="D175" t="s">
-        <v>339</v>
       </c>
       <c r="E175">
         <v>10</v>
@@ -14946,16 +14945,16 @@
     </row>
     <row r="176" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B176" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C176" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D176" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E176">
         <v>28</v>
@@ -15023,16 +15022,16 @@
     </row>
     <row r="177" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="B177" t="s">
+        <v>166</v>
+      </c>
+      <c r="C177" t="s">
+        <v>24</v>
+      </c>
+      <c r="D177" t="s">
         <v>341</v>
-      </c>
-      <c r="B177" t="s">
-        <v>167</v>
-      </c>
-      <c r="C177" t="s">
-        <v>25</v>
-      </c>
-      <c r="D177" t="s">
-        <v>342</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -15100,16 +15099,16 @@
     </row>
     <row r="178" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B178" t="s">
+        <v>55</v>
+      </c>
+      <c r="C178" t="s">
+        <v>24</v>
+      </c>
+      <c r="D178" t="s">
         <v>343</v>
-      </c>
-      <c r="B178" t="s">
-        <v>56</v>
-      </c>
-      <c r="C178" t="s">
-        <v>25</v>
-      </c>
-      <c r="D178" t="s">
-        <v>344</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -15177,16 +15176,16 @@
     </row>
     <row r="179" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A179" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B179" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C179" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D179" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E179">
         <v>9</v>
@@ -15254,16 +15253,16 @@
     </row>
     <row r="180" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B180" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C180" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D180" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -15331,16 +15330,16 @@
     </row>
     <row r="181" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="B181" t="s">
+        <v>191</v>
+      </c>
+      <c r="C181" t="s">
+        <v>29</v>
+      </c>
+      <c r="D181" t="s">
         <v>347</v>
-      </c>
-      <c r="B181" t="s">
-        <v>192</v>
-      </c>
-      <c r="C181" t="s">
-        <v>30</v>
-      </c>
-      <c r="D181" t="s">
-        <v>348</v>
       </c>
       <c r="E181">
         <v>12</v>
@@ -15408,16 +15407,16 @@
     </row>
     <row r="182" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B182" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C182" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D182" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E182">
         <v>12</v>
@@ -15485,16 +15484,16 @@
     </row>
     <row r="183" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A183" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B183" t="s">
+        <v>211</v>
+      </c>
+      <c r="C183" t="s">
+        <v>24</v>
+      </c>
+      <c r="D183" t="s">
         <v>350</v>
-      </c>
-      <c r="B183" t="s">
-        <v>212</v>
-      </c>
-      <c r="C183" t="s">
-        <v>25</v>
-      </c>
-      <c r="D183" t="s">
-        <v>351</v>
       </c>
       <c r="E183">
         <v>3</v>
@@ -15562,16 +15561,16 @@
     </row>
     <row r="184" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A184" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B184" t="s">
+        <v>37</v>
+      </c>
+      <c r="C184" t="s">
+        <v>24</v>
+      </c>
+      <c r="D184" t="s">
         <v>352</v>
-      </c>
-      <c r="B184" t="s">
-        <v>38</v>
-      </c>
-      <c r="C184" t="s">
-        <v>25</v>
-      </c>
-      <c r="D184" t="s">
-        <v>353</v>
       </c>
       <c r="E184">
         <v>15</v>
@@ -15639,16 +15638,16 @@
     </row>
     <row r="185" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A185" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="B185" t="s">
+        <v>166</v>
+      </c>
+      <c r="C185" t="s">
+        <v>24</v>
+      </c>
+      <c r="D185" t="s">
         <v>354</v>
-      </c>
-      <c r="B185" t="s">
-        <v>167</v>
-      </c>
-      <c r="C185" t="s">
-        <v>25</v>
-      </c>
-      <c r="D185" t="s">
-        <v>355</v>
       </c>
       <c r="E185">
         <v>2</v>
@@ -15716,16 +15715,16 @@
     </row>
     <row r="186" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A186" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B186" t="s">
+        <v>23</v>
+      </c>
+      <c r="C186" t="s">
         <v>24</v>
       </c>
-      <c r="C186" t="s">
-        <v>25</v>
-      </c>
       <c r="D186" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E186">
         <v>34</v>
@@ -15793,16 +15792,16 @@
     </row>
     <row r="187" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B187" t="s">
+        <v>166</v>
+      </c>
+      <c r="C187" t="s">
+        <v>24</v>
+      </c>
+      <c r="D187" t="s">
         <v>357</v>
-      </c>
-      <c r="B187" t="s">
-        <v>167</v>
-      </c>
-      <c r="C187" t="s">
-        <v>25</v>
-      </c>
-      <c r="D187" t="s">
-        <v>358</v>
       </c>
       <c r="E187">
         <v>2</v>
@@ -15870,16 +15869,16 @@
     </row>
     <row r="188" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A188" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B188" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C188" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D188" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E188">
         <v>7</v>
@@ -15947,16 +15946,16 @@
     </row>
     <row r="189" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A189" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B189" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C189" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D189" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E189">
         <v>4</v>
@@ -16024,16 +16023,16 @@
     </row>
     <row r="190" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A190" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B190" t="s">
+        <v>211</v>
+      </c>
+      <c r="C190" t="s">
+        <v>24</v>
+      </c>
+      <c r="D190" t="s">
         <v>361</v>
-      </c>
-      <c r="B190" t="s">
-        <v>212</v>
-      </c>
-      <c r="C190" t="s">
-        <v>25</v>
-      </c>
-      <c r="D190" t="s">
-        <v>362</v>
       </c>
       <c r="E190">
         <v>9</v>
@@ -16101,16 +16100,16 @@
     </row>
     <row r="191" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A191" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="B191" t="s">
+        <v>83</v>
+      </c>
+      <c r="C191" t="s">
+        <v>24</v>
+      </c>
+      <c r="D191" t="s">
         <v>363</v>
-      </c>
-      <c r="B191" t="s">
-        <v>84</v>
-      </c>
-      <c r="C191" t="s">
-        <v>25</v>
-      </c>
-      <c r="D191" t="s">
-        <v>364</v>
       </c>
       <c r="E191">
         <v>3</v>
@@ -16178,16 +16177,16 @@
     </row>
     <row r="192" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B192" t="s">
+        <v>191</v>
+      </c>
+      <c r="C192" t="s">
+        <v>29</v>
+      </c>
+      <c r="D192" t="s">
         <v>365</v>
-      </c>
-      <c r="B192" t="s">
-        <v>192</v>
-      </c>
-      <c r="C192" t="s">
-        <v>30</v>
-      </c>
-      <c r="D192" t="s">
-        <v>366</v>
       </c>
       <c r="E192">
         <v>6</v>
@@ -16255,16 +16254,16 @@
     </row>
     <row r="193" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A193" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B193" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C193" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D193" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E193">
         <v>9</v>
@@ -16332,16 +16331,16 @@
     </row>
     <row r="194" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A194" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B194" t="s">
+        <v>216</v>
+      </c>
+      <c r="C194" t="s">
+        <v>24</v>
+      </c>
+      <c r="D194" t="s">
         <v>368</v>
-      </c>
-      <c r="B194" t="s">
-        <v>217</v>
-      </c>
-      <c r="C194" t="s">
-        <v>25</v>
-      </c>
-      <c r="D194" t="s">
-        <v>369</v>
       </c>
       <c r="E194">
         <v>10</v>
@@ -16409,16 +16408,16 @@
     </row>
     <row r="195" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A195" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B195" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C195" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D195" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E195">
         <v>16</v>
@@ -16486,16 +16485,16 @@
     </row>
     <row r="196" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A196" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B196" t="s">
+        <v>216</v>
+      </c>
+      <c r="C196" t="s">
+        <v>24</v>
+      </c>
+      <c r="D196" t="s">
         <v>371</v>
-      </c>
-      <c r="B196" t="s">
-        <v>217</v>
-      </c>
-      <c r="C196" t="s">
-        <v>25</v>
-      </c>
-      <c r="D196" t="s">
-        <v>372</v>
       </c>
       <c r="E196">
         <v>20</v>
@@ -16563,16 +16562,16 @@
     </row>
     <row r="197" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A197" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B197" t="s">
         <v>373</v>
       </c>
-      <c r="B197" t="s">
+      <c r="C197" t="s">
+        <v>24</v>
+      </c>
+      <c r="D197" t="s">
         <v>374</v>
-      </c>
-      <c r="C197" t="s">
-        <v>25</v>
-      </c>
-      <c r="D197" t="s">
-        <v>375</v>
       </c>
       <c r="E197">
         <v>6</v>
@@ -16640,16 +16639,16 @@
     </row>
     <row r="198" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A198" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B198" t="s">
+        <v>58</v>
+      </c>
+      <c r="C198" t="s">
+        <v>24</v>
+      </c>
+      <c r="D198" t="s">
         <v>376</v>
-      </c>
-      <c r="B198" t="s">
-        <v>59</v>
-      </c>
-      <c r="C198" t="s">
-        <v>25</v>
-      </c>
-      <c r="D198" t="s">
-        <v>377</v>
       </c>
       <c r="E198">
         <v>3</v>
@@ -16717,16 +16716,16 @@
     </row>
     <row r="199" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A199" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B199" t="s">
+        <v>337</v>
+      </c>
+      <c r="C199" t="s">
+        <v>24</v>
+      </c>
+      <c r="D199" t="s">
         <v>378</v>
-      </c>
-      <c r="B199" t="s">
-        <v>338</v>
-      </c>
-      <c r="C199" t="s">
-        <v>25</v>
-      </c>
-      <c r="D199" t="s">
-        <v>379</v>
       </c>
       <c r="E199">
         <v>10</v>
@@ -16794,16 +16793,16 @@
     </row>
     <row r="200" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A200" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="B200" t="s">
+        <v>216</v>
+      </c>
+      <c r="C200" t="s">
+        <v>24</v>
+      </c>
+      <c r="D200" t="s">
         <v>380</v>
-      </c>
-      <c r="B200" t="s">
-        <v>217</v>
-      </c>
-      <c r="C200" t="s">
-        <v>25</v>
-      </c>
-      <c r="D200" t="s">
-        <v>381</v>
       </c>
       <c r="E200">
         <v>10</v>
@@ -16871,16 +16870,16 @@
     </row>
     <row r="201" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A201" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="B201" t="s">
+        <v>79</v>
+      </c>
+      <c r="C201" t="s">
+        <v>24</v>
+      </c>
+      <c r="D201" t="s">
         <v>382</v>
-      </c>
-      <c r="B201" t="s">
-        <v>80</v>
-      </c>
-      <c r="C201" t="s">
-        <v>25</v>
-      </c>
-      <c r="D201" t="s">
-        <v>383</v>
       </c>
       <c r="E201">
         <v>11</v>
@@ -16948,16 +16947,16 @@
     </row>
     <row r="202" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A202" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B202" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C202" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D202" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E202">
         <v>9</v>
@@ -17025,16 +17024,16 @@
     </row>
     <row r="203" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A203" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B203" t="s">
+        <v>334</v>
+      </c>
+      <c r="C203" t="s">
+        <v>24</v>
+      </c>
+      <c r="D203" t="s">
         <v>385</v>
-      </c>
-      <c r="B203" t="s">
-        <v>335</v>
-      </c>
-      <c r="C203" t="s">
-        <v>25</v>
-      </c>
-      <c r="D203" t="s">
-        <v>386</v>
       </c>
       <c r="E203">
         <v>4</v>
@@ -17102,16 +17101,16 @@
     </row>
     <row r="204" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A204" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="B204" t="s">
+        <v>334</v>
+      </c>
+      <c r="C204" t="s">
+        <v>24</v>
+      </c>
+      <c r="D204" t="s">
         <v>387</v>
-      </c>
-      <c r="B204" t="s">
-        <v>335</v>
-      </c>
-      <c r="C204" t="s">
-        <v>25</v>
-      </c>
-      <c r="D204" t="s">
-        <v>388</v>
       </c>
       <c r="E204">
         <v>5</v>

</xml_diff>

<commit_message>
alteração na planilha PV.xlsx
</commit_message>
<xml_diff>
--- a/PV.xlsx
+++ b/PV.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FCDE3D8-F520-400C-B9CB-0CA026209328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F36D56E-72B6-4BDB-A605-7E0EC70350B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="PV_ABRIL" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DadosExternos_1" localSheetId="0" hidden="1">PV_ABRIL!$A$1:$Y$195</definedName>
+    <definedName name="DadosExternos_1" localSheetId="0" hidden="1">PV_ABRIL!$A$1:$Y$188</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="145">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -387,9 +387,6 @@
   </si>
   <si>
     <t>HVHV308331-01</t>
-  </si>
-  <si>
-    <t>HVHV308331-02</t>
   </si>
   <si>
     <t>HVHV308716-01</t>
@@ -1350,8 +1347,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Follow_up" displayName="Follow_up" ref="A1:Y195" tableType="queryTable" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" tableBorderDxfId="26" totalsRowBorderDxfId="25">
-  <autoFilter ref="A1:Y195" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Follow_up" displayName="Follow_up" ref="A1:Y188" tableType="queryTable" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" tableBorderDxfId="26" totalsRowBorderDxfId="25">
+  <autoFilter ref="A1:Y188" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="25">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" uniqueName="1" name="PV" queryTableFieldId="1" dataDxfId="24"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" uniqueName="2" name="CLIENTE" queryTableFieldId="2" dataDxfId="23"/>
@@ -1646,7 +1643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y195"/>
+  <dimension ref="A1:Y188"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.5546875" style="1" customWidth="1"/>
@@ -10077,7 +10074,7 @@
         <v>25</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D110" s="8">
         <v>46137</v>
@@ -10154,7 +10151,7 @@
         <v>25</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D111" s="8">
         <v>46137</v>
@@ -12458,7 +12455,7 @@
     </row>
     <row r="141" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A141" s="6">
-        <v>6796</v>
+        <v>6798</v>
       </c>
       <c r="B141" s="7" t="s">
         <v>99</v>
@@ -12467,10 +12464,10 @@
         <v>114</v>
       </c>
       <c r="D141" s="8">
-        <v>46101</v>
+        <v>46122</v>
       </c>
       <c r="E141" s="9">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F141" s="9">
         <v>10</v>
@@ -12535,7 +12532,7 @@
     </row>
     <row r="142" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A142" s="6">
-        <v>6798</v>
+        <v>6797</v>
       </c>
       <c r="B142" s="7" t="s">
         <v>99</v>
@@ -12547,7 +12544,7 @@
         <v>46122</v>
       </c>
       <c r="E142" s="9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F142" s="9">
         <v>10</v>
@@ -12612,22 +12609,22 @@
     </row>
     <row r="143" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A143" s="6">
-        <v>6797</v>
+        <v>6830</v>
       </c>
       <c r="B143" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C143" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D143" s="8">
         <v>46122</v>
       </c>
       <c r="E143" s="9">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F143" s="9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G143" s="9">
         <v>0</v>
@@ -12648,7 +12645,7 @@
         <v>0</v>
       </c>
       <c r="M143" s="9">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N143" s="9">
         <v>0</v>
@@ -12657,7 +12654,7 @@
         <v>0</v>
       </c>
       <c r="P143" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q143" s="9">
         <v>6</v>
@@ -12669,10 +12666,10 @@
         <v>0</v>
       </c>
       <c r="T143" s="9">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="U143" s="9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="V143" s="9">
         <v>0</v>
@@ -12689,34 +12686,34 @@
     </row>
     <row r="144" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A144" s="6">
-        <v>6830</v>
+        <v>6767</v>
       </c>
       <c r="B144" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C144" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D144" s="8">
-        <v>46122</v>
+        <v>46127</v>
       </c>
       <c r="E144" s="9">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F144" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G144" s="9">
         <v>0</v>
       </c>
       <c r="H144" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I144" s="9">
         <v>0</v>
       </c>
       <c r="J144" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K144" s="9">
         <v>0</v>
@@ -12731,13 +12728,13 @@
         <v>0</v>
       </c>
       <c r="O144" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P144" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q144" s="9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R144" s="9">
         <v>0</v>
@@ -12746,7 +12743,7 @@
         <v>0</v>
       </c>
       <c r="T144" s="9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="U144" s="9">
         <v>5</v>
@@ -12766,7 +12763,7 @@
     </row>
     <row r="145" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A145" s="6">
-        <v>6803</v>
+        <v>6892</v>
       </c>
       <c r="B145" s="7" t="s">
         <v>99</v>
@@ -12775,25 +12772,25 @@
         <v>116</v>
       </c>
       <c r="D145" s="8">
-        <v>46108</v>
+        <v>46169</v>
       </c>
       <c r="E145" s="9">
+        <v>15</v>
+      </c>
+      <c r="F145" s="9">
+        <v>2</v>
+      </c>
+      <c r="G145" s="9">
+        <v>0</v>
+      </c>
+      <c r="H145" s="9">
         <v>3</v>
       </c>
-      <c r="F145" s="9">
-        <v>5</v>
-      </c>
-      <c r="G145" s="9">
-        <v>0</v>
-      </c>
-      <c r="H145" s="9">
-        <v>0</v>
-      </c>
       <c r="I145" s="9">
         <v>0</v>
       </c>
       <c r="J145" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K145" s="9">
         <v>0</v>
@@ -12808,13 +12805,13 @@
         <v>0</v>
       </c>
       <c r="O145" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P145" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q145" s="9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R145" s="9">
         <v>0</v>
@@ -12823,7 +12820,7 @@
         <v>0</v>
       </c>
       <c r="T145" s="9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="U145" s="9">
         <v>5</v>
@@ -12843,34 +12840,34 @@
     </row>
     <row r="146" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A146" s="6">
-        <v>6802</v>
+        <v>6828</v>
       </c>
       <c r="B146" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C146" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D146" s="8">
-        <v>46108</v>
+        <v>46127</v>
       </c>
       <c r="E146" s="9">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="F146" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G146" s="9">
         <v>0</v>
       </c>
       <c r="H146" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I146" s="9">
         <v>0</v>
       </c>
       <c r="J146" s="9">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K146" s="9">
         <v>0</v>
@@ -12879,7 +12876,7 @@
         <v>0</v>
       </c>
       <c r="M146" s="9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N146" s="9">
         <v>0</v>
@@ -12888,10 +12885,10 @@
         <v>0</v>
       </c>
       <c r="P146" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q146" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R146" s="9">
         <v>0</v>
@@ -12900,10 +12897,10 @@
         <v>0</v>
       </c>
       <c r="T146" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U146" s="9">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="V146" s="9">
         <v>0</v>
@@ -12920,7 +12917,7 @@
     </row>
     <row r="147" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A147" s="6">
-        <v>6767</v>
+        <v>6888</v>
       </c>
       <c r="B147" s="7" t="s">
         <v>99</v>
@@ -12929,25 +12926,25 @@
         <v>117</v>
       </c>
       <c r="D147" s="8">
-        <v>46127</v>
+        <v>46170</v>
       </c>
       <c r="E147" s="9">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="F147" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G147" s="9">
         <v>0</v>
       </c>
       <c r="H147" s="9">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="I147" s="9">
         <v>0</v>
       </c>
       <c r="J147" s="9">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="K147" s="9">
         <v>0</v>
@@ -12956,19 +12953,19 @@
         <v>0</v>
       </c>
       <c r="M147" s="9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N147" s="9">
         <v>0</v>
       </c>
       <c r="O147" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P147" s="9">
         <v>0</v>
       </c>
       <c r="Q147" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R147" s="9">
         <v>0</v>
@@ -12977,10 +12974,10 @@
         <v>0</v>
       </c>
       <c r="T147" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U147" s="9">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="V147" s="9">
         <v>0</v>
@@ -12997,34 +12994,34 @@
     </row>
     <row r="148" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A148" s="6">
-        <v>6892</v>
+        <v>6827</v>
       </c>
       <c r="B148" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C148" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D148" s="8">
-        <v>46169</v>
+        <v>46122</v>
       </c>
       <c r="E148" s="9">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F148" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G148" s="9">
         <v>0</v>
       </c>
       <c r="H148" s="9">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="I148" s="9">
         <v>0</v>
       </c>
       <c r="J148" s="9">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="K148" s="9">
         <v>0</v>
@@ -13039,13 +13036,13 @@
         <v>0</v>
       </c>
       <c r="O148" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P148" s="9">
         <v>0</v>
       </c>
       <c r="Q148" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R148" s="9">
         <v>0</v>
@@ -13054,10 +13051,10 @@
         <v>0</v>
       </c>
       <c r="T148" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U148" s="9">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="V148" s="9">
         <v>0</v>
@@ -13074,7 +13071,7 @@
     </row>
     <row r="149" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A149" s="6">
-        <v>6600</v>
+        <v>6800</v>
       </c>
       <c r="B149" s="7" t="s">
         <v>99</v>
@@ -13083,10 +13080,10 @@
         <v>118</v>
       </c>
       <c r="D149" s="8">
-        <v>46095</v>
+        <v>46151</v>
       </c>
       <c r="E149" s="9">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F149" s="9">
         <v>0</v>
@@ -13101,40 +13098,40 @@
         <v>0</v>
       </c>
       <c r="J149" s="9">
+        <v>60</v>
+      </c>
+      <c r="K149" s="9">
+        <v>0</v>
+      </c>
+      <c r="L149" s="9">
+        <v>0</v>
+      </c>
+      <c r="M149" s="9">
+        <v>10</v>
+      </c>
+      <c r="N149" s="9">
+        <v>0</v>
+      </c>
+      <c r="O149" s="9">
+        <v>0</v>
+      </c>
+      <c r="P149" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q149" s="9">
+        <v>5</v>
+      </c>
+      <c r="R149" s="9">
+        <v>0</v>
+      </c>
+      <c r="S149" s="9">
+        <v>0</v>
+      </c>
+      <c r="T149" s="9">
+        <v>0</v>
+      </c>
+      <c r="U149" s="9">
         <v>30</v>
-      </c>
-      <c r="K149" s="9">
-        <v>0</v>
-      </c>
-      <c r="L149" s="9">
-        <v>0</v>
-      </c>
-      <c r="M149" s="9">
-        <v>5</v>
-      </c>
-      <c r="N149" s="9">
-        <v>0</v>
-      </c>
-      <c r="O149" s="9">
-        <v>0</v>
-      </c>
-      <c r="P149" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q149" s="9">
-        <v>5</v>
-      </c>
-      <c r="R149" s="9">
-        <v>0</v>
-      </c>
-      <c r="S149" s="9">
-        <v>0</v>
-      </c>
-      <c r="T149" s="9">
-        <v>0</v>
-      </c>
-      <c r="U149" s="9">
-        <v>15</v>
       </c>
       <c r="V149" s="9">
         <v>0</v>
@@ -13151,7 +13148,7 @@
     </row>
     <row r="150" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A150" s="6">
-        <v>6828</v>
+        <v>6984</v>
       </c>
       <c r="B150" s="7" t="s">
         <v>99</v>
@@ -13160,10 +13157,10 @@
         <v>118</v>
       </c>
       <c r="D150" s="8">
-        <v>46127</v>
+        <v>46177</v>
       </c>
       <c r="E150" s="9">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="F150" s="9">
         <v>0</v>
@@ -13178,40 +13175,40 @@
         <v>0</v>
       </c>
       <c r="J150" s="9">
+        <v>60</v>
+      </c>
+      <c r="K150" s="9">
+        <v>0</v>
+      </c>
+      <c r="L150" s="9">
+        <v>0</v>
+      </c>
+      <c r="M150" s="9">
+        <v>10</v>
+      </c>
+      <c r="N150" s="9">
+        <v>0</v>
+      </c>
+      <c r="O150" s="9">
+        <v>0</v>
+      </c>
+      <c r="P150" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q150" s="9">
+        <v>5</v>
+      </c>
+      <c r="R150" s="9">
+        <v>0</v>
+      </c>
+      <c r="S150" s="9">
+        <v>0</v>
+      </c>
+      <c r="T150" s="9">
+        <v>0</v>
+      </c>
+      <c r="U150" s="9">
         <v>30</v>
-      </c>
-      <c r="K150" s="9">
-        <v>0</v>
-      </c>
-      <c r="L150" s="9">
-        <v>0</v>
-      </c>
-      <c r="M150" s="9">
-        <v>5</v>
-      </c>
-      <c r="N150" s="9">
-        <v>0</v>
-      </c>
-      <c r="O150" s="9">
-        <v>0</v>
-      </c>
-      <c r="P150" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q150" s="9">
-        <v>5</v>
-      </c>
-      <c r="R150" s="9">
-        <v>0</v>
-      </c>
-      <c r="S150" s="9">
-        <v>0</v>
-      </c>
-      <c r="T150" s="9">
-        <v>0</v>
-      </c>
-      <c r="U150" s="9">
-        <v>15</v>
       </c>
       <c r="V150" s="9">
         <v>0</v>
@@ -13228,55 +13225,55 @@
     </row>
     <row r="151" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A151" s="6">
-        <v>6888</v>
+        <v>6780</v>
       </c>
       <c r="B151" s="7" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="C151" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D151" s="8">
-        <v>46170</v>
+        <v>46113</v>
       </c>
       <c r="E151" s="9">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="F151" s="9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G151" s="9">
         <v>0</v>
       </c>
       <c r="H151" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I151" s="9">
         <v>0</v>
       </c>
       <c r="J151" s="9">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K151" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L151" s="9">
         <v>0</v>
       </c>
       <c r="M151" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N151" s="9">
         <v>0</v>
       </c>
       <c r="O151" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="P151" s="9">
         <v>0</v>
       </c>
       <c r="Q151" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R151" s="9">
         <v>0</v>
@@ -13288,7 +13285,7 @@
         <v>0</v>
       </c>
       <c r="U151" s="9">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="V151" s="9">
         <v>0</v>
@@ -13305,55 +13302,55 @@
     </row>
     <row r="152" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A152" s="6">
-        <v>6827</v>
+        <v>6879</v>
       </c>
       <c r="B152" s="7" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="C152" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D152" s="8">
-        <v>46122</v>
+        <v>46171</v>
       </c>
       <c r="E152" s="9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F152" s="9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G152" s="9">
         <v>0</v>
       </c>
       <c r="H152" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I152" s="9">
         <v>0</v>
       </c>
       <c r="J152" s="9">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="K152" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L152" s="9">
         <v>0</v>
       </c>
       <c r="M152" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N152" s="9">
         <v>0</v>
       </c>
       <c r="O152" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="P152" s="9">
         <v>0</v>
       </c>
       <c r="Q152" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R152" s="9">
         <v>0</v>
@@ -13365,7 +13362,7 @@
         <v>0</v>
       </c>
       <c r="U152" s="9">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="V152" s="9">
         <v>0</v>
@@ -13382,55 +13379,55 @@
     </row>
     <row r="153" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A153" s="6">
-        <v>6800</v>
+        <v>6859</v>
       </c>
       <c r="B153" s="7" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="C153" s="7" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D153" s="8">
-        <v>46151</v>
+        <v>46125</v>
       </c>
       <c r="E153" s="9">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F153" s="9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G153" s="9">
         <v>0</v>
       </c>
       <c r="H153" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I153" s="9">
         <v>0</v>
       </c>
       <c r="J153" s="9">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="K153" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L153" s="9">
         <v>0</v>
       </c>
       <c r="M153" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N153" s="9">
         <v>0</v>
       </c>
       <c r="O153" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="P153" s="9">
         <v>0</v>
       </c>
       <c r="Q153" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R153" s="9">
         <v>0</v>
@@ -13442,7 +13439,7 @@
         <v>0</v>
       </c>
       <c r="U153" s="9">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="V153" s="9">
         <v>0</v>
@@ -13459,34 +13456,34 @@
     </row>
     <row r="154" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A154" s="6">
-        <v>6984</v>
+        <v>6814</v>
       </c>
       <c r="B154" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C154" s="7" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D154" s="8">
-        <v>46177</v>
+        <v>46129</v>
       </c>
       <c r="E154" s="9">
         <v>3</v>
       </c>
       <c r="F154" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G154" s="9">
         <v>0</v>
       </c>
       <c r="H154" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I154" s="9">
         <v>0</v>
       </c>
       <c r="J154" s="9">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="K154" s="9">
         <v>0</v>
@@ -13507,7 +13504,7 @@
         <v>0</v>
       </c>
       <c r="Q154" s="9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R154" s="9">
         <v>0</v>
@@ -13516,10 +13513,10 @@
         <v>0</v>
       </c>
       <c r="T154" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U154" s="9">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="V154" s="9">
         <v>0</v>
@@ -13536,22 +13533,22 @@
     </row>
     <row r="155" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A155" s="6">
-        <v>6780</v>
+        <v>6839</v>
       </c>
       <c r="B155" s="7" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="C155" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D155" s="8">
-        <v>46113</v>
+        <v>46134</v>
       </c>
       <c r="E155" s="9">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="F155" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G155" s="9">
         <v>0</v>
@@ -13566,25 +13563,25 @@
         <v>0</v>
       </c>
       <c r="K155" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L155" s="9">
         <v>0</v>
       </c>
       <c r="M155" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N155" s="9">
         <v>0</v>
       </c>
       <c r="O155" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P155" s="9">
         <v>0</v>
       </c>
       <c r="Q155" s="9">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R155" s="9">
         <v>0</v>
@@ -13593,7 +13590,7 @@
         <v>0</v>
       </c>
       <c r="T155" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U155" s="9">
         <v>10</v>
@@ -13613,22 +13610,22 @@
     </row>
     <row r="156" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A156" s="6">
-        <v>6879</v>
+        <v>6815</v>
       </c>
       <c r="B156" s="7" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="C156" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D156" s="8">
-        <v>46171</v>
+        <v>46163</v>
       </c>
       <c r="E156" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F156" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G156" s="9">
         <v>0</v>
@@ -13643,25 +13640,25 @@
         <v>0</v>
       </c>
       <c r="K156" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L156" s="9">
         <v>0</v>
       </c>
       <c r="M156" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N156" s="9">
         <v>0</v>
       </c>
       <c r="O156" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P156" s="9">
         <v>0</v>
       </c>
       <c r="Q156" s="9">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R156" s="9">
         <v>0</v>
@@ -13670,7 +13667,7 @@
         <v>0</v>
       </c>
       <c r="T156" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U156" s="9">
         <v>10</v>
@@ -13690,56 +13687,56 @@
     </row>
     <row r="157" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A157" s="6">
-        <v>6859</v>
+        <v>6816</v>
       </c>
       <c r="B157" s="7" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="C157" s="7" t="s">
         <v>122</v>
       </c>
       <c r="D157" s="8">
-        <v>46125</v>
+        <v>46170</v>
       </c>
       <c r="E157" s="9">
+        <v>2</v>
+      </c>
+      <c r="F157" s="9">
+        <v>5</v>
+      </c>
+      <c r="G157" s="9">
+        <v>0</v>
+      </c>
+      <c r="H157" s="9">
+        <v>0</v>
+      </c>
+      <c r="I157" s="9">
+        <v>0</v>
+      </c>
+      <c r="J157" s="9">
+        <v>0</v>
+      </c>
+      <c r="K157" s="9">
+        <v>0</v>
+      </c>
+      <c r="L157" s="9">
+        <v>0</v>
+      </c>
+      <c r="M157" s="9">
+        <v>10</v>
+      </c>
+      <c r="N157" s="9">
+        <v>0</v>
+      </c>
+      <c r="O157" s="9">
+        <v>0</v>
+      </c>
+      <c r="P157" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q157" s="9">
         <v>6</v>
       </c>
-      <c r="F157" s="9">
-        <v>2</v>
-      </c>
-      <c r="G157" s="9">
-        <v>0</v>
-      </c>
-      <c r="H157" s="9">
-        <v>0</v>
-      </c>
-      <c r="I157" s="9">
-        <v>0</v>
-      </c>
-      <c r="J157" s="9">
-        <v>0</v>
-      </c>
-      <c r="K157" s="9">
-        <v>10</v>
-      </c>
-      <c r="L157" s="9">
-        <v>0</v>
-      </c>
-      <c r="M157" s="9">
-        <v>0</v>
-      </c>
-      <c r="N157" s="9">
-        <v>0</v>
-      </c>
-      <c r="O157" s="9">
-        <v>15</v>
-      </c>
-      <c r="P157" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q157" s="9">
-        <v>0</v>
-      </c>
       <c r="R157" s="9">
         <v>0</v>
       </c>
@@ -13747,7 +13744,7 @@
         <v>0</v>
       </c>
       <c r="T157" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U157" s="9">
         <v>10</v>
@@ -13767,19 +13764,19 @@
     </row>
     <row r="158" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A158" s="6">
-        <v>6814</v>
+        <v>6817</v>
       </c>
       <c r="B158" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C158" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D158" s="8">
-        <v>46129</v>
+        <v>46171</v>
       </c>
       <c r="E158" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F158" s="9">
         <v>5</v>
@@ -13844,22 +13841,22 @@
     </row>
     <row r="159" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A159" s="6">
-        <v>6839</v>
+        <v>6710</v>
       </c>
       <c r="B159" s="7" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="C159" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D159" s="8">
-        <v>46134</v>
+        <v>46118</v>
       </c>
       <c r="E159" s="9">
-        <v>3</v>
+        <v>146</v>
       </c>
       <c r="F159" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G159" s="9">
         <v>0</v>
@@ -13877,10 +13874,10 @@
         <v>0</v>
       </c>
       <c r="L159" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="M159" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N159" s="9">
         <v>0</v>
@@ -13892,7 +13889,7 @@
         <v>0</v>
       </c>
       <c r="Q159" s="9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R159" s="9">
         <v>0</v>
@@ -13901,13 +13898,13 @@
         <v>0</v>
       </c>
       <c r="T159" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U159" s="9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="V159" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W159" s="9">
         <v>0</v>
@@ -13921,19 +13918,19 @@
     </row>
     <row r="160" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A160" s="6">
-        <v>6815</v>
+        <v>6878</v>
       </c>
       <c r="B160" s="7" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="C160" s="7" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D160" s="8">
-        <v>46163</v>
+        <v>46151</v>
       </c>
       <c r="E160" s="9">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="F160" s="9">
         <v>5</v>
@@ -13951,25 +13948,25 @@
         <v>0</v>
       </c>
       <c r="K160" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L160" s="9">
         <v>0</v>
       </c>
       <c r="M160" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N160" s="9">
         <v>0</v>
       </c>
       <c r="O160" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="P160" s="9">
         <v>0</v>
       </c>
       <c r="Q160" s="9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R160" s="9">
         <v>0</v>
@@ -13978,10 +13975,10 @@
         <v>0</v>
       </c>
       <c r="T160" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U160" s="9">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="V160" s="9">
         <v>0</v>
@@ -13998,25 +13995,25 @@
     </row>
     <row r="161" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A161" s="6">
-        <v>6816</v>
+        <v>6549</v>
       </c>
       <c r="B161" s="7" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="C161" s="7" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D161" s="8">
-        <v>46170</v>
+        <v>46113</v>
       </c>
       <c r="E161" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F161" s="9">
-        <v>5</v>
+        <v>400</v>
       </c>
       <c r="G161" s="9">
-        <v>0</v>
+        <v>680</v>
       </c>
       <c r="H161" s="9">
         <v>0</v>
@@ -14034,7 +14031,7 @@
         <v>0</v>
       </c>
       <c r="M161" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N161" s="9">
         <v>0</v>
@@ -14046,7 +14043,7 @@
         <v>0</v>
       </c>
       <c r="Q161" s="9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R161" s="9">
         <v>0</v>
@@ -14055,16 +14052,16 @@
         <v>0</v>
       </c>
       <c r="T161" s="9">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="U161" s="9">
-        <v>10</v>
+        <v>240</v>
       </c>
       <c r="V161" s="9">
         <v>0</v>
       </c>
       <c r="W161" s="9">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="X161" s="9">
         <v>0</v>
@@ -14075,25 +14072,25 @@
     </row>
     <row r="162" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A162" s="6">
-        <v>6817</v>
+        <v>6550</v>
       </c>
       <c r="B162" s="7" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="C162" s="7" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D162" s="8">
-        <v>46171</v>
+        <v>46118</v>
       </c>
       <c r="E162" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F162" s="9">
-        <v>5</v>
+        <v>400</v>
       </c>
       <c r="G162" s="9">
-        <v>0</v>
+        <v>680</v>
       </c>
       <c r="H162" s="9">
         <v>0</v>
@@ -14111,7 +14108,7 @@
         <v>0</v>
       </c>
       <c r="M162" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N162" s="9">
         <v>0</v>
@@ -14123,7 +14120,7 @@
         <v>0</v>
       </c>
       <c r="Q162" s="9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R162" s="9">
         <v>0</v>
@@ -14132,16 +14129,16 @@
         <v>0</v>
       </c>
       <c r="T162" s="9">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="U162" s="9">
-        <v>10</v>
+        <v>240</v>
       </c>
       <c r="V162" s="9">
         <v>0</v>
       </c>
       <c r="W162" s="9">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="X162" s="9">
         <v>0</v>
@@ -14152,25 +14149,25 @@
     </row>
     <row r="163" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A163" s="6">
-        <v>6710</v>
+        <v>6547</v>
       </c>
       <c r="B163" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C163" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D163" s="8">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="E163" s="9">
-        <v>146</v>
+        <v>1</v>
       </c>
       <c r="F163" s="9">
-        <v>2</v>
+        <v>400</v>
       </c>
       <c r="G163" s="9">
-        <v>0</v>
+        <v>680</v>
       </c>
       <c r="H163" s="9">
         <v>0</v>
@@ -14185,7 +14182,7 @@
         <v>0</v>
       </c>
       <c r="L163" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="M163" s="9">
         <v>0</v>
@@ -14209,16 +14206,16 @@
         <v>0</v>
       </c>
       <c r="T163" s="9">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="U163" s="9">
-        <v>5</v>
+        <v>240</v>
       </c>
       <c r="V163" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W163" s="9">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="X163" s="9">
         <v>0</v>
@@ -14229,25 +14226,25 @@
     </row>
     <row r="164" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A164" s="6">
-        <v>6878</v>
+        <v>6548</v>
       </c>
       <c r="B164" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C164" s="7" t="s">
         <v>126</v>
       </c>
       <c r="D164" s="8">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="E164" s="9">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="F164" s="9">
-        <v>5</v>
+        <v>400</v>
       </c>
       <c r="G164" s="9">
-        <v>0</v>
+        <v>680</v>
       </c>
       <c r="H164" s="9">
         <v>0</v>
@@ -14259,7 +14256,7 @@
         <v>0</v>
       </c>
       <c r="K164" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L164" s="9">
         <v>0</v>
@@ -14271,7 +14268,7 @@
         <v>0</v>
       </c>
       <c r="O164" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P164" s="9">
         <v>0</v>
@@ -14286,16 +14283,16 @@
         <v>0</v>
       </c>
       <c r="T164" s="9">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="U164" s="9">
-        <v>15</v>
+        <v>240</v>
       </c>
       <c r="V164" s="9">
         <v>0</v>
       </c>
       <c r="W164" s="9">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="X164" s="9">
         <v>0</v>
@@ -14306,10 +14303,10 @@
     </row>
     <row r="165" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A165" s="6">
-        <v>6549</v>
+        <v>6552</v>
       </c>
       <c r="B165" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C165" s="7" t="s">
         <v>127</v>
@@ -14383,10 +14380,10 @@
     </row>
     <row r="166" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A166" s="6">
-        <v>6550</v>
+        <v>6553</v>
       </c>
       <c r="B166" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C166" s="7" t="s">
         <v>127</v>
@@ -14460,10 +14457,10 @@
     </row>
     <row r="167" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A167" s="6">
-        <v>6547</v>
+        <v>6554</v>
       </c>
       <c r="B167" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C167" s="7" t="s">
         <v>127</v>
@@ -14537,10 +14534,10 @@
     </row>
     <row r="168" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A168" s="6">
-        <v>6548</v>
+        <v>6555</v>
       </c>
       <c r="B168" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C168" s="7" t="s">
         <v>127</v>
@@ -14614,25 +14611,25 @@
     </row>
     <row r="169" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A169" s="6">
-        <v>6552</v>
+        <v>6942</v>
       </c>
       <c r="B169" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C169" s="7" t="s">
         <v>128</v>
       </c>
       <c r="D169" s="8">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="E169" s="9">
         <v>1</v>
       </c>
       <c r="F169" s="9">
-        <v>400</v>
+        <v>2</v>
       </c>
       <c r="G169" s="9">
-        <v>680</v>
+        <v>0</v>
       </c>
       <c r="H169" s="9">
         <v>0</v>
@@ -14647,7 +14644,7 @@
         <v>0</v>
       </c>
       <c r="L169" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M169" s="9">
         <v>0</v>
@@ -14671,16 +14668,16 @@
         <v>0</v>
       </c>
       <c r="T169" s="9">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="U169" s="9">
-        <v>240</v>
+        <v>3</v>
       </c>
       <c r="V169" s="9">
         <v>0</v>
       </c>
       <c r="W169" s="9">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="X169" s="9">
         <v>0</v>
@@ -14691,25 +14688,25 @@
     </row>
     <row r="170" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A170" s="6">
-        <v>6553</v>
+        <v>6953</v>
       </c>
       <c r="B170" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C170" s="7" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="D170" s="8">
-        <v>46118</v>
+        <v>46121</v>
       </c>
       <c r="E170" s="9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F170" s="9">
-        <v>400</v>
+        <v>5</v>
       </c>
       <c r="G170" s="9">
-        <v>680</v>
+        <v>0</v>
       </c>
       <c r="H170" s="9">
         <v>0</v>
@@ -14724,7 +14721,7 @@
         <v>0</v>
       </c>
       <c r="L170" s="9">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M170" s="9">
         <v>0</v>
@@ -14748,16 +14745,16 @@
         <v>0</v>
       </c>
       <c r="T170" s="9">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="U170" s="9">
-        <v>240</v>
+        <v>5</v>
       </c>
       <c r="V170" s="9">
         <v>0</v>
       </c>
       <c r="W170" s="9">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="X170" s="9">
         <v>0</v>
@@ -14768,25 +14765,25 @@
     </row>
     <row r="171" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A171" s="6">
-        <v>6554</v>
+        <v>6882</v>
       </c>
       <c r="B171" s="7" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C171" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D171" s="8">
-        <v>46128</v>
+        <v>46165</v>
       </c>
       <c r="E171" s="9">
         <v>1</v>
       </c>
       <c r="F171" s="9">
-        <v>400</v>
+        <v>2</v>
       </c>
       <c r="G171" s="9">
-        <v>680</v>
+        <v>0</v>
       </c>
       <c r="H171" s="9">
         <v>0</v>
@@ -14795,7 +14792,7 @@
         <v>0</v>
       </c>
       <c r="J171" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K171" s="9">
         <v>0</v>
@@ -14825,16 +14822,16 @@
         <v>0</v>
       </c>
       <c r="T171" s="9">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="U171" s="9">
-        <v>240</v>
+        <v>8</v>
       </c>
       <c r="V171" s="9">
         <v>0</v>
       </c>
       <c r="W171" s="9">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="X171" s="9">
         <v>0</v>
@@ -14845,25 +14842,25 @@
     </row>
     <row r="172" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A172" s="6">
-        <v>6555</v>
+        <v>6960</v>
       </c>
       <c r="B172" s="7" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C172" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D172" s="8">
-        <v>46153</v>
+        <v>46165</v>
       </c>
       <c r="E172" s="9">
         <v>1</v>
       </c>
       <c r="F172" s="9">
-        <v>400</v>
+        <v>2</v>
       </c>
       <c r="G172" s="9">
-        <v>680</v>
+        <v>0</v>
       </c>
       <c r="H172" s="9">
         <v>0</v>
@@ -14872,7 +14869,7 @@
         <v>0</v>
       </c>
       <c r="J172" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K172" s="9">
         <v>0</v>
@@ -14902,16 +14899,16 @@
         <v>0</v>
       </c>
       <c r="T172" s="9">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="U172" s="9">
-        <v>240</v>
+        <v>8</v>
       </c>
       <c r="V172" s="9">
         <v>0</v>
       </c>
       <c r="W172" s="9">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="X172" s="9">
         <v>0</v>
@@ -14922,22 +14919,22 @@
     </row>
     <row r="173" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A173" s="6">
-        <v>6942</v>
+        <v>6955</v>
       </c>
       <c r="B173" s="7" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C173" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D173" s="8">
-        <v>46123</v>
+        <v>46146</v>
       </c>
       <c r="E173" s="9">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F173" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G173" s="9">
         <v>0</v>
@@ -14999,28 +14996,28 @@
     </row>
     <row r="174" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A174" s="6">
-        <v>6953</v>
+        <v>6637</v>
       </c>
       <c r="B174" s="7" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C174" s="7" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="D174" s="8">
-        <v>46121</v>
+        <v>46135</v>
       </c>
       <c r="E174" s="9">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F174" s="9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G174" s="9">
         <v>0</v>
       </c>
       <c r="H174" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I174" s="9">
         <v>0</v>
@@ -15032,10 +15029,10 @@
         <v>0</v>
       </c>
       <c r="L174" s="9">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M174" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N174" s="9">
         <v>0</v>
@@ -15056,10 +15053,10 @@
         <v>0</v>
       </c>
       <c r="T174" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U174" s="9">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="V174" s="9">
         <v>0</v>
@@ -15076,34 +15073,34 @@
     </row>
     <row r="175" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A175" s="6">
-        <v>6882</v>
+        <v>6845</v>
       </c>
       <c r="B175" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C175" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D175" s="8">
-        <v>46165</v>
+        <v>46189</v>
       </c>
       <c r="E175" s="9">
+        <v>10</v>
+      </c>
+      <c r="F175" s="9">
         <v>1</v>
       </c>
-      <c r="F175" s="9">
-        <v>2</v>
-      </c>
       <c r="G175" s="9">
         <v>0</v>
       </c>
       <c r="H175" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I175" s="9">
         <v>0</v>
       </c>
       <c r="J175" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K175" s="9">
         <v>0</v>
@@ -15112,7 +15109,7 @@
         <v>0</v>
       </c>
       <c r="M175" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N175" s="9">
         <v>0</v>
@@ -15133,10 +15130,10 @@
         <v>0</v>
       </c>
       <c r="T175" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U175" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V175" s="9">
         <v>0</v>
@@ -15153,34 +15150,34 @@
     </row>
     <row r="176" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A176" s="6">
-        <v>6960</v>
+        <v>6883</v>
       </c>
       <c r="B176" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C176" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D176" s="8">
-        <v>46165</v>
+        <v>46196</v>
       </c>
       <c r="E176" s="9">
+        <v>20</v>
+      </c>
+      <c r="F176" s="9">
         <v>1</v>
       </c>
-      <c r="F176" s="9">
-        <v>2</v>
-      </c>
       <c r="G176" s="9">
         <v>0</v>
       </c>
       <c r="H176" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I176" s="9">
         <v>0</v>
       </c>
       <c r="J176" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K176" s="9">
         <v>0</v>
@@ -15189,7 +15186,7 @@
         <v>0</v>
       </c>
       <c r="M176" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N176" s="9">
         <v>0</v>
@@ -15210,10 +15207,10 @@
         <v>0</v>
       </c>
       <c r="T176" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U176" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V176" s="9">
         <v>0</v>
@@ -15230,7 +15227,7 @@
     </row>
     <row r="177" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A177" s="6">
-        <v>6955</v>
+        <v>6949</v>
       </c>
       <c r="B177" s="7" t="s">
         <v>99</v>
@@ -15239,19 +15236,19 @@
         <v>131</v>
       </c>
       <c r="D177" s="8">
-        <v>46146</v>
+        <v>46202</v>
       </c>
       <c r="E177" s="9">
         <v>10</v>
       </c>
       <c r="F177" s="9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G177" s="9">
         <v>0</v>
       </c>
       <c r="H177" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I177" s="9">
         <v>0</v>
@@ -15263,10 +15260,10 @@
         <v>0</v>
       </c>
       <c r="L177" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M177" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N177" s="9">
         <v>0</v>
@@ -15287,10 +15284,10 @@
         <v>0</v>
       </c>
       <c r="T177" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U177" s="9">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="V177" s="9">
         <v>0</v>
@@ -15307,19 +15304,19 @@
     </row>
     <row r="178" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A178" s="6">
-        <v>6637</v>
+        <v>6954</v>
       </c>
       <c r="B178" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C178" s="7" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="D178" s="8">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="E178" s="9">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="F178" s="9">
         <v>1</v>
@@ -15328,7 +15325,7 @@
         <v>0</v>
       </c>
       <c r="H178" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I178" s="9">
         <v>0</v>
@@ -15337,19 +15334,19 @@
         <v>0</v>
       </c>
       <c r="K178" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L178" s="9">
         <v>0</v>
       </c>
       <c r="M178" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N178" s="9">
         <v>0</v>
       </c>
       <c r="O178" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P178" s="9">
         <v>0</v>
@@ -15364,10 +15361,10 @@
         <v>0</v>
       </c>
       <c r="T178" s="9">
-        <v>5</v>
+        <v>0.25</v>
       </c>
       <c r="U178" s="9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V178" s="9">
         <v>0</v>
@@ -15384,7 +15381,7 @@
     </row>
     <row r="179" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A179" s="6">
-        <v>6845</v>
+        <v>6846</v>
       </c>
       <c r="B179" s="7" t="s">
         <v>99</v>
@@ -15393,25 +15390,25 @@
         <v>132</v>
       </c>
       <c r="D179" s="8">
-        <v>46189</v>
+        <v>46132</v>
       </c>
       <c r="E179" s="9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F179" s="9">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G179" s="9">
         <v>0</v>
       </c>
       <c r="H179" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I179" s="9">
         <v>0</v>
       </c>
       <c r="J179" s="9">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K179" s="9">
         <v>0</v>
@@ -15420,7 +15417,7 @@
         <v>0</v>
       </c>
       <c r="M179" s="9">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="N179" s="9">
         <v>0</v>
@@ -15441,10 +15438,10 @@
         <v>0</v>
       </c>
       <c r="T179" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U179" s="9">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="V179" s="9">
         <v>0</v>
@@ -15461,7 +15458,7 @@
     </row>
     <row r="180" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A180" s="6">
-        <v>6883</v>
+        <v>6941</v>
       </c>
       <c r="B180" s="7" t="s">
         <v>99</v>
@@ -15470,25 +15467,25 @@
         <v>132</v>
       </c>
       <c r="D180" s="8">
-        <v>46196</v>
+        <v>46135</v>
       </c>
       <c r="E180" s="9">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F180" s="9">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G180" s="9">
         <v>0</v>
       </c>
       <c r="H180" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I180" s="9">
         <v>0</v>
       </c>
       <c r="J180" s="9">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K180" s="9">
         <v>0</v>
@@ -15497,7 +15494,7 @@
         <v>0</v>
       </c>
       <c r="M180" s="9">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="N180" s="9">
         <v>0</v>
@@ -15518,10 +15515,10 @@
         <v>0</v>
       </c>
       <c r="T180" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U180" s="9">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="V180" s="9">
         <v>0</v>
@@ -15538,28 +15535,28 @@
     </row>
     <row r="181" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A181" s="6">
-        <v>6949</v>
+        <v>6799</v>
       </c>
       <c r="B181" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C181" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D181" s="8">
-        <v>46202</v>
+        <v>46132</v>
       </c>
       <c r="E181" s="9">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F181" s="9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G181" s="9">
         <v>0</v>
       </c>
       <c r="H181" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I181" s="9">
         <v>0</v>
@@ -15574,13 +15571,13 @@
         <v>0</v>
       </c>
       <c r="M181" s="9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N181" s="9">
         <v>0</v>
       </c>
       <c r="O181" s="9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P181" s="9">
         <v>0</v>
@@ -15595,10 +15592,10 @@
         <v>0</v>
       </c>
       <c r="T181" s="9">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="U181" s="9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V181" s="9">
         <v>0</v>
@@ -15615,22 +15612,22 @@
     </row>
     <row r="182" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A182" s="6">
-        <v>6954</v>
+        <v>6831</v>
       </c>
       <c r="B182" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C182" s="7" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="D182" s="8">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="E182" s="9">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="F182" s="9">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G182" s="9">
         <v>0</v>
@@ -15645,19 +15642,19 @@
         <v>0</v>
       </c>
       <c r="K182" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L182" s="9">
         <v>0</v>
       </c>
       <c r="M182" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N182" s="9">
         <v>0</v>
       </c>
       <c r="O182" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P182" s="9">
         <v>0</v>
@@ -15672,7 +15669,7 @@
         <v>0</v>
       </c>
       <c r="T182" s="9">
-        <v>0.25</v>
+        <v>15</v>
       </c>
       <c r="U182" s="9">
         <v>10</v>
@@ -15692,22 +15689,22 @@
     </row>
     <row r="183" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A183" s="6">
-        <v>6685</v>
+        <v>6829</v>
       </c>
       <c r="B183" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C183" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D183" s="8">
-        <v>46106</v>
+        <v>46154</v>
       </c>
       <c r="E183" s="9">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F183" s="9">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G183" s="9">
         <v>0</v>
@@ -15719,7 +15716,7 @@
         <v>0</v>
       </c>
       <c r="J183" s="9">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K183" s="9">
         <v>0</v>
@@ -15728,7 +15725,7 @@
         <v>0</v>
       </c>
       <c r="M183" s="9">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="N183" s="9">
         <v>0</v>
@@ -15749,10 +15746,10 @@
         <v>0</v>
       </c>
       <c r="T183" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="U183" s="9">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="V183" s="9">
         <v>0</v>
@@ -15769,56 +15766,56 @@
     </row>
     <row r="184" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A184" s="6">
-        <v>6768</v>
+        <v>6784</v>
       </c>
       <c r="B184" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C184" s="7" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D184" s="8">
-        <v>46106</v>
+        <v>46135</v>
       </c>
       <c r="E184" s="9">
+        <v>200</v>
+      </c>
+      <c r="F184" s="9">
+        <v>1</v>
+      </c>
+      <c r="G184" s="9">
+        <v>0</v>
+      </c>
+      <c r="H184" s="9">
+        <v>0</v>
+      </c>
+      <c r="I184" s="9">
+        <v>0</v>
+      </c>
+      <c r="J184" s="9">
+        <v>0</v>
+      </c>
+      <c r="K184" s="9">
+        <v>0</v>
+      </c>
+      <c r="L184" s="9">
+        <v>0</v>
+      </c>
+      <c r="M184" s="9">
+        <v>3</v>
+      </c>
+      <c r="N184" s="9">
+        <v>0</v>
+      </c>
+      <c r="O184" s="9">
+        <v>0</v>
+      </c>
+      <c r="P184" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q184" s="9">
         <v>2</v>
       </c>
-      <c r="F184" s="9">
-        <v>10</v>
-      </c>
-      <c r="G184" s="9">
-        <v>0</v>
-      </c>
-      <c r="H184" s="9">
-        <v>0</v>
-      </c>
-      <c r="I184" s="9">
-        <v>0</v>
-      </c>
-      <c r="J184" s="9">
-        <v>30</v>
-      </c>
-      <c r="K184" s="9">
-        <v>0</v>
-      </c>
-      <c r="L184" s="9">
-        <v>0</v>
-      </c>
-      <c r="M184" s="9">
-        <v>60</v>
-      </c>
-      <c r="N184" s="9">
-        <v>0</v>
-      </c>
-      <c r="O184" s="9">
-        <v>0</v>
-      </c>
-      <c r="P184" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q184" s="9">
-        <v>0</v>
-      </c>
       <c r="R184" s="9">
         <v>0</v>
       </c>
@@ -15829,7 +15826,7 @@
         <v>0</v>
       </c>
       <c r="U184" s="9">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="V184" s="9">
         <v>0</v>
@@ -15846,23 +15843,23 @@
     </row>
     <row r="185" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A185" s="6">
-        <v>6785</v>
+        <v>6770</v>
       </c>
       <c r="B185" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C185" s="7" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D185" s="8">
-        <v>46108</v>
+        <v>46127</v>
       </c>
       <c r="E185" s="9">
+        <v>62</v>
+      </c>
+      <c r="F185" s="9">
         <v>3</v>
       </c>
-      <c r="F185" s="9">
-        <v>10</v>
-      </c>
       <c r="G185" s="9">
         <v>0</v>
       </c>
@@ -15873,7 +15870,7 @@
         <v>0</v>
       </c>
       <c r="J185" s="9">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K185" s="9">
         <v>0</v>
@@ -15882,7 +15879,7 @@
         <v>0</v>
       </c>
       <c r="M185" s="9">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="N185" s="9">
         <v>0</v>
@@ -15906,7 +15903,7 @@
         <v>0</v>
       </c>
       <c r="U185" s="9">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="V185" s="9">
         <v>0</v>
@@ -15923,34 +15920,34 @@
     </row>
     <row r="186" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A186" s="6">
-        <v>6846</v>
+        <v>6983</v>
       </c>
       <c r="B186" s="7" t="s">
-        <v>99</v>
+        <v>23</v>
       </c>
       <c r="C186" s="7" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="D186" s="8">
-        <v>46132</v>
+        <v>46127</v>
       </c>
       <c r="E186" s="9">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F186" s="9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G186" s="9">
         <v>0</v>
       </c>
       <c r="H186" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I186" s="9">
         <v>0</v>
       </c>
       <c r="J186" s="9">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K186" s="9">
         <v>0</v>
@@ -15959,7 +15956,7 @@
         <v>0</v>
       </c>
       <c r="M186" s="9">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="N186" s="9">
         <v>0</v>
@@ -15983,7 +15980,7 @@
         <v>0</v>
       </c>
       <c r="U186" s="9">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="V186" s="9">
         <v>0</v>
@@ -16000,616 +15997,77 @@
     </row>
     <row r="187" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A187" s="6">
-        <v>6941</v>
+        <v>6897</v>
       </c>
       <c r="B187" s="7" t="s">
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="C187" s="7" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="D187" s="8">
-        <v>46135</v>
+        <v>46125</v>
       </c>
       <c r="E187" s="9">
-        <v>1</v>
-      </c>
-      <c r="F187" s="9">
-        <v>10</v>
-      </c>
-      <c r="G187" s="9">
-        <v>0</v>
-      </c>
-      <c r="H187" s="9">
-        <v>0</v>
-      </c>
-      <c r="I187" s="9">
-        <v>0</v>
-      </c>
-      <c r="J187" s="9">
-        <v>30</v>
-      </c>
-      <c r="K187" s="9">
-        <v>0</v>
-      </c>
-      <c r="L187" s="9">
-        <v>0</v>
-      </c>
-      <c r="M187" s="9">
-        <v>60</v>
-      </c>
-      <c r="N187" s="9">
-        <v>0</v>
-      </c>
-      <c r="O187" s="9">
-        <v>0</v>
-      </c>
-      <c r="P187" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q187" s="9">
-        <v>0</v>
-      </c>
-      <c r="R187" s="9">
-        <v>0</v>
-      </c>
-      <c r="S187" s="9">
-        <v>0</v>
-      </c>
-      <c r="T187" s="9">
-        <v>0</v>
-      </c>
-      <c r="U187" s="9">
-        <v>25</v>
-      </c>
-      <c r="V187" s="9">
-        <v>0</v>
-      </c>
-      <c r="W187" s="9">
-        <v>0</v>
-      </c>
-      <c r="X187" s="9">
-        <v>0</v>
-      </c>
-      <c r="Y187" s="10">
-        <v>0</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="F187" s="9"/>
+      <c r="G187" s="9"/>
+      <c r="H187" s="9"/>
+      <c r="I187" s="9"/>
+      <c r="J187" s="9"/>
+      <c r="K187" s="9"/>
+      <c r="L187" s="9"/>
+      <c r="M187" s="9"/>
+      <c r="N187" s="9"/>
+      <c r="O187" s="9"/>
+      <c r="P187" s="9"/>
+      <c r="Q187" s="9"/>
+      <c r="R187" s="9"/>
+      <c r="S187" s="9"/>
+      <c r="T187" s="9"/>
+      <c r="U187" s="9"/>
+      <c r="V187" s="9"/>
+      <c r="W187" s="9"/>
+      <c r="X187" s="9"/>
+      <c r="Y187" s="10"/>
     </row>
     <row r="188" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A188" s="6">
-        <v>6799</v>
-      </c>
-      <c r="B188" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C188" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="D188" s="8">
+      <c r="A188" s="11">
+        <v>6912</v>
+      </c>
+      <c r="B188" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C188" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="D188" s="13">
         <v>46132</v>
       </c>
-      <c r="E188" s="9">
-        <v>3</v>
-      </c>
-      <c r="F188" s="9">
-        <v>5</v>
-      </c>
-      <c r="G188" s="9">
-        <v>0</v>
-      </c>
-      <c r="H188" s="9">
-        <v>0</v>
-      </c>
-      <c r="I188" s="9">
-        <v>0</v>
-      </c>
-      <c r="J188" s="9">
-        <v>0</v>
-      </c>
-      <c r="K188" s="9">
-        <v>0</v>
-      </c>
-      <c r="L188" s="9">
-        <v>0</v>
-      </c>
-      <c r="M188" s="9">
-        <v>10</v>
-      </c>
-      <c r="N188" s="9">
-        <v>0</v>
-      </c>
-      <c r="O188" s="9">
-        <v>5</v>
-      </c>
-      <c r="P188" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q188" s="9">
-        <v>0</v>
-      </c>
-      <c r="R188" s="9">
-        <v>0</v>
-      </c>
-      <c r="S188" s="9">
-        <v>0</v>
-      </c>
-      <c r="T188" s="9">
-        <v>20</v>
-      </c>
-      <c r="U188" s="9">
-        <v>10</v>
-      </c>
-      <c r="V188" s="9">
-        <v>0</v>
-      </c>
-      <c r="W188" s="9">
-        <v>0</v>
-      </c>
-      <c r="X188" s="9">
-        <v>0</v>
-      </c>
-      <c r="Y188" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="189" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A189" s="6">
-        <v>6831</v>
-      </c>
-      <c r="B189" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C189" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="D189" s="8">
-        <v>46142</v>
-      </c>
-      <c r="E189" s="9">
-        <v>9</v>
-      </c>
-      <c r="F189" s="9">
-        <v>15</v>
-      </c>
-      <c r="G189" s="9">
-        <v>0</v>
-      </c>
-      <c r="H189" s="9">
-        <v>0</v>
-      </c>
-      <c r="I189" s="9">
-        <v>0</v>
-      </c>
-      <c r="J189" s="9">
-        <v>0</v>
-      </c>
-      <c r="K189" s="9">
-        <v>0</v>
-      </c>
-      <c r="L189" s="9">
-        <v>0</v>
-      </c>
-      <c r="M189" s="9">
-        <v>10</v>
-      </c>
-      <c r="N189" s="9">
-        <v>0</v>
-      </c>
-      <c r="O189" s="9">
-        <v>0</v>
-      </c>
-      <c r="P189" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q189" s="9">
-        <v>0</v>
-      </c>
-      <c r="R189" s="9">
-        <v>0</v>
-      </c>
-      <c r="S189" s="9">
-        <v>0</v>
-      </c>
-      <c r="T189" s="9">
-        <v>15</v>
-      </c>
-      <c r="U189" s="9">
-        <v>10</v>
-      </c>
-      <c r="V189" s="9">
-        <v>0</v>
-      </c>
-      <c r="W189" s="9">
-        <v>0</v>
-      </c>
-      <c r="X189" s="9">
-        <v>0</v>
-      </c>
-      <c r="Y189" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="190" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A190" s="6">
-        <v>6829</v>
-      </c>
-      <c r="B190" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C190" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="D190" s="8">
-        <v>46154</v>
-      </c>
-      <c r="E190" s="9">
-        <v>6</v>
-      </c>
-      <c r="F190" s="9">
-        <v>15</v>
-      </c>
-      <c r="G190" s="9">
-        <v>0</v>
-      </c>
-      <c r="H190" s="9">
-        <v>0</v>
-      </c>
-      <c r="I190" s="9">
-        <v>0</v>
-      </c>
-      <c r="J190" s="9">
-        <v>0</v>
-      </c>
-      <c r="K190" s="9">
-        <v>0</v>
-      </c>
-      <c r="L190" s="9">
-        <v>0</v>
-      </c>
-      <c r="M190" s="9">
-        <v>10</v>
-      </c>
-      <c r="N190" s="9">
-        <v>0</v>
-      </c>
-      <c r="O190" s="9">
-        <v>0</v>
-      </c>
-      <c r="P190" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q190" s="9">
-        <v>0</v>
-      </c>
-      <c r="R190" s="9">
-        <v>0</v>
-      </c>
-      <c r="S190" s="9">
-        <v>0</v>
-      </c>
-      <c r="T190" s="9">
-        <v>15</v>
-      </c>
-      <c r="U190" s="9">
-        <v>10</v>
-      </c>
-      <c r="V190" s="9">
-        <v>0</v>
-      </c>
-      <c r="W190" s="9">
-        <v>0</v>
-      </c>
-      <c r="X190" s="9">
-        <v>0</v>
-      </c>
-      <c r="Y190" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="191" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A191" s="6">
-        <v>6784</v>
-      </c>
-      <c r="B191" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C191" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="D191" s="8">
-        <v>46135</v>
-      </c>
-      <c r="E191" s="9">
-        <v>200</v>
-      </c>
-      <c r="F191" s="9">
-        <v>1</v>
-      </c>
-      <c r="G191" s="9">
-        <v>0</v>
-      </c>
-      <c r="H191" s="9">
-        <v>0</v>
-      </c>
-      <c r="I191" s="9">
-        <v>0</v>
-      </c>
-      <c r="J191" s="9">
-        <v>0</v>
-      </c>
-      <c r="K191" s="9">
-        <v>0</v>
-      </c>
-      <c r="L191" s="9">
-        <v>0</v>
-      </c>
-      <c r="M191" s="9">
-        <v>3</v>
-      </c>
-      <c r="N191" s="9">
-        <v>0</v>
-      </c>
-      <c r="O191" s="9">
-        <v>0</v>
-      </c>
-      <c r="P191" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q191" s="9">
-        <v>2</v>
-      </c>
-      <c r="R191" s="9">
-        <v>0</v>
-      </c>
-      <c r="S191" s="9">
-        <v>0</v>
-      </c>
-      <c r="T191" s="9">
-        <v>0</v>
-      </c>
-      <c r="U191" s="9">
-        <v>1</v>
-      </c>
-      <c r="V191" s="9">
-        <v>0</v>
-      </c>
-      <c r="W191" s="9">
-        <v>0</v>
-      </c>
-      <c r="X191" s="9">
-        <v>0</v>
-      </c>
-      <c r="Y191" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="192" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A192" s="6">
-        <v>6770</v>
-      </c>
-      <c r="B192" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C192" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="D192" s="8">
-        <v>46127</v>
-      </c>
-      <c r="E192" s="9">
-        <v>62</v>
-      </c>
-      <c r="F192" s="9">
-        <v>3</v>
-      </c>
-      <c r="G192" s="9">
-        <v>0</v>
-      </c>
-      <c r="H192" s="9">
-        <v>0</v>
-      </c>
-      <c r="I192" s="9">
-        <v>0</v>
-      </c>
-      <c r="J192" s="9">
-        <v>5</v>
-      </c>
-      <c r="K192" s="9">
-        <v>0</v>
-      </c>
-      <c r="L192" s="9">
-        <v>0</v>
-      </c>
-      <c r="M192" s="9">
-        <v>0</v>
-      </c>
-      <c r="N192" s="9">
-        <v>0</v>
-      </c>
-      <c r="O192" s="9">
-        <v>0</v>
-      </c>
-      <c r="P192" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q192" s="9">
-        <v>0</v>
-      </c>
-      <c r="R192" s="9">
-        <v>0</v>
-      </c>
-      <c r="S192" s="9">
-        <v>0</v>
-      </c>
-      <c r="T192" s="9">
-        <v>0</v>
-      </c>
-      <c r="U192" s="9">
-        <v>2</v>
-      </c>
-      <c r="V192" s="9">
-        <v>0</v>
-      </c>
-      <c r="W192" s="9">
-        <v>0</v>
-      </c>
-      <c r="X192" s="9">
-        <v>0</v>
-      </c>
-      <c r="Y192" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="193" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A193" s="6">
-        <v>6983</v>
-      </c>
-      <c r="B193" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C193" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="D193" s="8">
-        <v>46127</v>
-      </c>
-      <c r="E193" s="9">
-        <v>1</v>
-      </c>
-      <c r="F193" s="9">
-        <v>0</v>
-      </c>
-      <c r="G193" s="9">
-        <v>0</v>
-      </c>
-      <c r="H193" s="9">
-        <v>3</v>
-      </c>
-      <c r="I193" s="9">
-        <v>0</v>
-      </c>
-      <c r="J193" s="9">
-        <v>0</v>
-      </c>
-      <c r="K193" s="9">
-        <v>0</v>
-      </c>
-      <c r="L193" s="9">
-        <v>0</v>
-      </c>
-      <c r="M193" s="9">
-        <v>0</v>
-      </c>
-      <c r="N193" s="9">
-        <v>0</v>
-      </c>
-      <c r="O193" s="9">
-        <v>0</v>
-      </c>
-      <c r="P193" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q193" s="9">
-        <v>0</v>
-      </c>
-      <c r="R193" s="9">
-        <v>0</v>
-      </c>
-      <c r="S193" s="9">
-        <v>0</v>
-      </c>
-      <c r="T193" s="9">
-        <v>0</v>
-      </c>
-      <c r="U193" s="9">
-        <v>3</v>
-      </c>
-      <c r="V193" s="9">
-        <v>0</v>
-      </c>
-      <c r="W193" s="9">
-        <v>0</v>
-      </c>
-      <c r="X193" s="9">
-        <v>0</v>
-      </c>
-      <c r="Y193" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="194" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A194" s="6">
-        <v>6897</v>
-      </c>
-      <c r="B194" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C194" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="D194" s="8">
-        <v>46125</v>
-      </c>
-      <c r="E194" s="9">
-        <v>6</v>
-      </c>
-      <c r="F194" s="9"/>
-      <c r="G194" s="9"/>
-      <c r="H194" s="9"/>
-      <c r="I194" s="9"/>
-      <c r="J194" s="9"/>
-      <c r="K194" s="9"/>
-      <c r="L194" s="9"/>
-      <c r="M194" s="9"/>
-      <c r="N194" s="9"/>
-      <c r="O194" s="9"/>
-      <c r="P194" s="9"/>
-      <c r="Q194" s="9"/>
-      <c r="R194" s="9"/>
-      <c r="S194" s="9"/>
-      <c r="T194" s="9"/>
-      <c r="U194" s="9"/>
-      <c r="V194" s="9"/>
-      <c r="W194" s="9"/>
-      <c r="X194" s="9"/>
-      <c r="Y194" s="10"/>
-    </row>
-    <row r="195" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A195" s="11">
-        <v>6912</v>
-      </c>
-      <c r="B195" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C195" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="D195" s="13">
-        <v>46132</v>
-      </c>
-      <c r="E195" s="14">
-        <v>10</v>
-      </c>
-      <c r="F195" s="14"/>
-      <c r="G195" s="14"/>
-      <c r="H195" s="14"/>
-      <c r="I195" s="14"/>
-      <c r="J195" s="14"/>
-      <c r="K195" s="14"/>
-      <c r="L195" s="14"/>
-      <c r="M195" s="14"/>
-      <c r="N195" s="14"/>
-      <c r="O195" s="14"/>
-      <c r="P195" s="14"/>
-      <c r="Q195" s="14"/>
-      <c r="R195" s="14"/>
-      <c r="S195" s="14"/>
-      <c r="T195" s="14"/>
-      <c r="U195" s="14"/>
-      <c r="V195" s="14"/>
-      <c r="W195" s="14"/>
-      <c r="X195" s="14"/>
-      <c r="Y195" s="15"/>
+      <c r="E188" s="14">
+        <v>10</v>
+      </c>
+      <c r="F188" s="14"/>
+      <c r="G188" s="14"/>
+      <c r="H188" s="14"/>
+      <c r="I188" s="14"/>
+      <c r="J188" s="14"/>
+      <c r="K188" s="14"/>
+      <c r="L188" s="14"/>
+      <c r="M188" s="14"/>
+      <c r="N188" s="14"/>
+      <c r="O188" s="14"/>
+      <c r="P188" s="14"/>
+      <c r="Q188" s="14"/>
+      <c r="R188" s="14"/>
+      <c r="S188" s="14"/>
+      <c r="T188" s="14"/>
+      <c r="U188" s="14"/>
+      <c r="V188" s="14"/>
+      <c r="W188" s="14"/>
+      <c r="X188" s="14"/>
+      <c r="Y188" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
acerto de tempos no roteiro de fabricação da planilha PV.xlsx
</commit_message>
<xml_diff>
--- a/PV.xlsx
+++ b/PV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F36D56E-72B6-4BDB-A605-7E0EC70350B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{031DFADB-86B9-4BDF-97CE-35E0D907DB1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="PV_ABRIL" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DadosExternos_1" localSheetId="0" hidden="1">PV_ABRIL!$A$1:$Y$188</definedName>
+    <definedName name="DadosExternos_1" localSheetId="0" hidden="1">PV_ABRIL!$A$1:$Y$189</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -626,7 +626,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -661,6 +661,14 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1347,8 +1355,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Follow_up" displayName="Follow_up" ref="A1:Y188" tableType="queryTable" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" tableBorderDxfId="26" totalsRowBorderDxfId="25">
-  <autoFilter ref="A1:Y188" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Follow_up" displayName="Follow_up" ref="A1:Y189" tableType="queryTable" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" tableBorderDxfId="26" totalsRowBorderDxfId="25">
+  <autoFilter ref="A1:Y189" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="25">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" uniqueName="1" name="PV" queryTableFieldId="1" dataDxfId="24"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" uniqueName="2" name="CLIENTE" queryTableFieldId="2" dataDxfId="23"/>
@@ -1643,7 +1651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y188"/>
+  <dimension ref="A1:Y189"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.5546875" style="1" customWidth="1"/>
@@ -16011,26 +16019,66 @@
       <c r="E187" s="9">
         <v>6</v>
       </c>
-      <c r="F187" s="9"/>
-      <c r="G187" s="9"/>
-      <c r="H187" s="9"/>
-      <c r="I187" s="9"/>
-      <c r="J187" s="9"/>
-      <c r="K187" s="9"/>
-      <c r="L187" s="9"/>
-      <c r="M187" s="9"/>
-      <c r="N187" s="9"/>
-      <c r="O187" s="9"/>
-      <c r="P187" s="9"/>
-      <c r="Q187" s="9"/>
-      <c r="R187" s="9"/>
-      <c r="S187" s="9"/>
-      <c r="T187" s="9"/>
-      <c r="U187" s="9"/>
-      <c r="V187" s="9"/>
-      <c r="W187" s="9"/>
-      <c r="X187" s="9"/>
-      <c r="Y187" s="10"/>
+      <c r="F187" s="9">
+        <v>0</v>
+      </c>
+      <c r="G187" s="9">
+        <v>0</v>
+      </c>
+      <c r="H187" s="9">
+        <v>5</v>
+      </c>
+      <c r="I187" s="9">
+        <v>0</v>
+      </c>
+      <c r="J187" s="9">
+        <v>0</v>
+      </c>
+      <c r="K187" s="9">
+        <v>0</v>
+      </c>
+      <c r="L187" s="9">
+        <v>0</v>
+      </c>
+      <c r="M187" s="9">
+        <v>0</v>
+      </c>
+      <c r="N187" s="9">
+        <v>0</v>
+      </c>
+      <c r="O187" s="9">
+        <v>0</v>
+      </c>
+      <c r="P187" s="9">
+        <v>10</v>
+      </c>
+      <c r="Q187" s="9">
+        <v>0</v>
+      </c>
+      <c r="R187" s="9">
+        <v>0</v>
+      </c>
+      <c r="S187" s="9">
+        <v>0</v>
+      </c>
+      <c r="T187" s="9">
+        <v>0</v>
+      </c>
+      <c r="U187" s="9">
+        <v>5</v>
+      </c>
+      <c r="V187" s="9">
+        <v>0</v>
+      </c>
+      <c r="W187" s="9">
+        <v>0</v>
+      </c>
+      <c r="X187" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y187" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="188" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A188" s="11">
@@ -16048,26 +16096,93 @@
       <c r="E188" s="14">
         <v>10</v>
       </c>
-      <c r="F188" s="14"/>
-      <c r="G188" s="14"/>
-      <c r="H188" s="14"/>
-      <c r="I188" s="14"/>
-      <c r="J188" s="14"/>
-      <c r="K188" s="14"/>
-      <c r="L188" s="14"/>
-      <c r="M188" s="14"/>
-      <c r="N188" s="14"/>
-      <c r="O188" s="14"/>
-      <c r="P188" s="14"/>
-      <c r="Q188" s="14"/>
-      <c r="R188" s="14"/>
-      <c r="S188" s="14"/>
-      <c r="T188" s="14"/>
-      <c r="U188" s="14"/>
-      <c r="V188" s="14"/>
-      <c r="W188" s="14"/>
-      <c r="X188" s="14"/>
-      <c r="Y188" s="15"/>
+      <c r="F188" s="14">
+        <v>2</v>
+      </c>
+      <c r="G188" s="14">
+        <v>0</v>
+      </c>
+      <c r="H188" s="14">
+        <v>0</v>
+      </c>
+      <c r="I188" s="14">
+        <v>0</v>
+      </c>
+      <c r="J188" s="14">
+        <v>0</v>
+      </c>
+      <c r="K188" s="14">
+        <v>0</v>
+      </c>
+      <c r="L188" s="14">
+        <v>0</v>
+      </c>
+      <c r="M188" s="14">
+        <v>5</v>
+      </c>
+      <c r="N188" s="14">
+        <v>0</v>
+      </c>
+      <c r="O188" s="14">
+        <v>0</v>
+      </c>
+      <c r="P188" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q188" s="14">
+        <v>0</v>
+      </c>
+      <c r="R188" s="14">
+        <v>0</v>
+      </c>
+      <c r="S188" s="14">
+        <v>0</v>
+      </c>
+      <c r="T188" s="14">
+        <v>0</v>
+      </c>
+      <c r="U188" s="14">
+        <v>2</v>
+      </c>
+      <c r="V188" s="14">
+        <v>0</v>
+      </c>
+      <c r="W188" s="14">
+        <v>0</v>
+      </c>
+      <c r="X188" s="14">
+        <v>0</v>
+      </c>
+      <c r="Y188" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A189" s="16"/>
+      <c r="B189" s="17"/>
+      <c r="C189" s="17"/>
+      <c r="D189" s="13"/>
+      <c r="E189" s="18"/>
+      <c r="F189" s="18"/>
+      <c r="G189" s="18"/>
+      <c r="H189" s="18"/>
+      <c r="I189" s="18"/>
+      <c r="J189" s="18"/>
+      <c r="K189" s="18"/>
+      <c r="L189" s="18"/>
+      <c r="M189" s="18"/>
+      <c r="N189" s="18"/>
+      <c r="O189" s="18"/>
+      <c r="P189" s="18"/>
+      <c r="Q189" s="18"/>
+      <c r="R189" s="18"/>
+      <c r="S189" s="18"/>
+      <c r="T189" s="18"/>
+      <c r="U189" s="18"/>
+      <c r="V189" s="18"/>
+      <c r="W189" s="18"/>
+      <c r="X189" s="18"/>
+      <c r="Y189" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
exclui arquivo word e inclui arquivo excel INDICADOR_PROVEDORES.xlsx na pasta Indicadores_Compras_Fornecedores
</commit_message>
<xml_diff>
--- a/PV.xlsx
+++ b/PV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65C08C2B-5071-4081-861A-ECD2314BA864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F4BE580-B1F2-456B-8BC1-47E190589189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,10 +18,21 @@
   <definedNames>
     <definedName name="DadosExternos_1" localSheetId="0" hidden="1">Planilha1!$A$1:$Z$220</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>

</xml_diff>